<commit_message>
V2 Reimplementation: first iteration (V1 final backup only)
</commit_message>
<xml_diff>
--- a/data/benchmark_specification_matrix.xlsx
+++ b/data/benchmark_specification_matrix.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Benchmark Spec Matrix" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Topic Allocation (Locked)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmark Spec Matrix" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topic Allocation (Locked)" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -43,30 +43,8 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
-    <font>
-      <name val="Arial Unicode MS"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="1"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="1"/>
-      <family val="2"/>
-      <i val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -77,6 +55,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF305496"/>
         <bgColor rgb="FF666699"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -92,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -110,6 +94,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -371,7 +359,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P109"/>
+  <dimension ref="A1:P151"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1219,7 +1207,7 @@
       </c>
       <c r="P10" s="1" t="inlineStr">
         <is>
-          <t>Had to add a backslash in answer output. The reasoning was fine, but the model hallucinated</t>
+          <t>Had to add a backslash in answer output. The reasoning was fine, but the model hallucinated | AUDIT (2026-08): re-verified by direct execution during T1-T3 validation pass -- code now correctly raises SyntaxError exactly as claimed, corrected snippet parses and runs. This item's fix (above) was already applied; no further change needed.</t>
         </is>
       </c>
     </row>
@@ -2174,7 +2162,7 @@
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>The following Python function is intended to return a string describing a 2‑D point using the structural pattern‑matching features described in the context. However, the code contains a subtle bug that causes a `NameError` when the point lies on the Y‑axis (e.g., `(0, 5)`). Analyze the match‑case structure, identify the exact line and operator/identifier that is incorrect, and provide the corrected version of that line.
+          <t>The following Python function is intended to return a string describing a 2‑D point using the structural pattern‑matching features described in the context. However, the code contains a subtle bug that causes a `UnboundLocalError` when the point lies on the Y‑axis (e.g., `(0, 5)`). Analyze the match‑case structure, identify the exact line and operator/identifier that is incorrect, and provide the corrected version of that line.
 ```python
 def describe_point(point):
     match point:
@@ -2193,7 +2181,7 @@
       </c>
       <c r="L21" s="4" t="inlineStr">
         <is>
-          <t>The bug is on the line `return f"Y={x}"` inside the `case (0, y):` block. In this pattern the variable bound from the subject is `y`, not `x`; `x` is undefined here, leading to a `NameError`. The corrected line should use the bound variable `y`:
+          <t>The bug is on the line `return f"Y={x}"` inside the `case (0, y):` block. In this pattern the variable bound from the subject is `y`, not `x`; `x` is undefined here, leading to a `UnboundLocalError`. The corrected line should use the bound variable `y`:
 ```python
         case (0, y):
             return f"Y={y}"
@@ -2215,7 +2203,11 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="P21" s="1" t="n"/>
+      <c r="P21" s="1" t="inlineStr">
+        <is>
+          <t>it gives UnboundLocalError when actually got executed the LLM gave NameError</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="307" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
@@ -5112,7 +5104,7 @@
       </c>
       <c r="M51" s="4" t="inlineStr">
         <is>
-          <t>topic_4_modules.pdf_26</t>
+          <t>topic_4_modules.pdf_27</t>
         </is>
       </c>
       <c r="N51" s="4" t="inlineStr">
@@ -5125,7 +5117,11 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="P51" s="4" t="n"/>
+      <c r="P51" s="4" t="inlineStr">
+        <is>
+          <t>AUDIT (2026-08): pulled the actual PDF chunks. Supporting_Chunks pointed at topic_4_modules.pdf_26, which is only the tail of a dir(builtins) name list plus the bare heading '6.4. Packages' -- no definition text. The real definition ("Packages are a way of structuring Python's module namespace...") is in chunk 27. Fixed Supporting_Chunks to topic_4_modules.pdf_27. Reference_Answer text was already accurate, unchanged.</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="43" customFormat="1" customHeight="1" s="8">
       <c r="A52" s="7" t="inlineStr">
@@ -6277,7 +6273,7 @@
       </c>
       <c r="M64" s="4" t="inlineStr">
         <is>
-          <t>topic_5_input_output.pdf_17</t>
+          <t>topic_5_input_output.pdf_16</t>
         </is>
       </c>
       <c r="N64" s="4" t="inlineStr">
@@ -6290,7 +6286,11 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="P64" s="4" t="n"/>
+      <c r="P64" s="4" t="inlineStr">
+        <is>
+          <t>AUDIT (2026-08): pulled the actual PDF chunks. Supporting_Chunks pointed at topic_5_input_output.pdf_17, which covers %-style formatting and the start of open() -- no mention of zfill() anywhere. The exact zfill() examples quoted in the answer ('12'.zfill(5), '-3.14'.zfill(7), etc.) are verbatim in chunk 16. Fixed Supporting_Chunks to topic_5_input_output.pdf_16 (off-by-one). Reference_Answer text was already accurate, unchanged.</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="225" customFormat="1" customHeight="1" s="8">
       <c r="A65" s="7" t="inlineStr">
@@ -6746,7 +6746,7 @@
       </c>
       <c r="P69" s="4" t="inlineStr">
         <is>
-          <t>changed to NameError instead of Syntax in "the interpreter sees an incomplete statement and raises a ``NameError`"</t>
+          <t>changed to NameError instead of Syntax in "the interpreter sees an incomplete statement and raises a ``NameError`" | AUDIT (2026-08): re-verified by direct execution during T4-T6 validation pass -- code now correctly raises NameError exactly as claimed. This item's fix (above) was already applied; no further change needed.</t>
         </is>
       </c>
     </row>
@@ -9682,7 +9682,7 @@
       </c>
       <c r="P99" s="4" t="n"/>
     </row>
-    <row r="100" customFormat="1" s="8">
+    <row r="100" ht="225" customFormat="1" customHeight="1" s="8">
       <c r="A100" s="7" t="inlineStr">
         <is>
           <t>T7_012</t>
@@ -9730,13 +9730,49 @@
       </c>
       <c r="J100" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="K100" s="4" t="n"/>
-      <c r="L100" s="4" t="n"/>
-      <c r="M100" s="4" t="n"/>
-      <c r="N100" s="4" t="n"/>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K100" s="4" t="inlineStr">
+        <is>
+          <t>The following Python code defines a custom iterator class intended to produce the sequence of integers from 0 up to (but not including) a given limit. However, when you run the loop `for n in Counter(3): print(n)`, the output is `1 2 3 4` instead of the expected `0 1 2`. Identify the exact line that contains the bug, explain why it causes the off‑by‑one error, and provide the corrected version of that line (or the whole method if you prefer). 
+```python
+class Counter:
+    def __init__(self, limit):
+        self.limit = limit
+        self.current = 0
+    def __iter__(self):
+        return self
+    def __next__(self):
+        if self.current &lt;= self.limit:
+            self.current += 1
+            return self.current
+        else:
+            raise StopIteration
+```</t>
+        </is>
+      </c>
+      <c r="L100" s="4" t="inlineStr">
+        <is>
+          <t>The bug is in the `__next__` method, specifically the line `self.current += 1` that occurs **before** the value is returned. Because `self.current` starts at 0, the method increments it to 1 and then returns 1 on the first call, so the sequence starts at 1 and runs one step past the intended limit (the `&lt;=` test also allows the extra value). To produce 0‑based values and stop before `limit`, either return the current value first and then increment, or adjust the condition. A minimal fix is to change the two lines inside the `if` block to:
+```python
+            result = self.current
+            self.current += 1
+            return result
+```
+Alternatively, you could keep the return‑first style and change the condition to `if self.current &lt; self.limit:` with the original increment‑after‑return logic. Either correction stops the iterator after yielding 0, 1, 2 for `limit=3`.</t>
+        </is>
+      </c>
+      <c r="M100" s="4" t="inlineStr">
+        <is>
+          <t>topic_7_oop.pdf_52, topic_7_oop.pdf_53, topic_7_oop.pdf_54</t>
+        </is>
+      </c>
+      <c r="N100" s="4" t="inlineStr">
+        <is>
+          <t>Custom iterator implementation</t>
+        </is>
+      </c>
       <c r="O100" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
@@ -9849,7 +9885,7 @@
       </c>
       <c r="P101" s="4" t="n"/>
     </row>
-    <row r="102" ht="409.6" customFormat="1" customHeight="1" s="8">
+    <row r="102" ht="409.5" customFormat="1" customHeight="1" s="8">
       <c r="A102" s="7" t="inlineStr">
         <is>
           <t>T7_014</t>
@@ -10127,13 +10163,28 @@
       </c>
       <c r="K104" s="4" t="inlineStr">
         <is>
-          <t>Below are two class definitions that each provide a way to make a method that returns the string 'hello world'.\n\nSnippet A (method defined inside the class):\n```python\nclass A:\n    def greet(self):\n        return 'hello world'\n```\n\nSnippet B (function defined outside and assigned as a class attribute):\n```python\ndef external_greet(self):\n    return 'hello world'\n\nclass B:\n    greet = external_greet\n```\n\nBoth classes are instantiated as `a = A()` and `b = B()`.\n\n**Task:** Analyse and compare the two approaches. Specifically, break down how the method objects are created and bound to instances, how the `self` argument is supplied when `a.greet()` and `b.greet()` are called, and discuss any differences in readability, convention adherence, and potential sources of confusion that stem from the technique shown in Snippet B. Use only the concepts presented in the context.</t>
+          <t>Below are two class definitions that each provide a way to make a method that returns the string 'hello world'.
+Snippet A (method defined inside the class):
+```python
+class A:
+    def greet(self):
+        return 'hello world'
+```
+Snippet B (function defined outside and assigned as a class attribute):
+```python
+def external_greet(self):
+    return 'hello world'
+class B:
+    greet = external_greet
+```
+Both classes are instantiated as `a = A()` and `b = B()`.
+**Task:** Analyse and compare the two approaches. Specifically, break down how the method objects are created and bound to instances, how the `self` argument is supplied when `a.greet()` and `b.greet()` are called, and discuss any differences in readability, convention adherence, and potential sources of confusion that stem from the technique shown in Snippet B. Use only the concepts presented in the context.</t>
         </is>
       </c>
       <c r="L104" s="4" t="inlineStr">
         <is>
           <t>In Snippet A the method `greet` is defined directly inside the class body; Python automatically creates a function object and, when accessed through an instance (`a.greet`), wraps it in a bound method that supplies the instance as the first argument (`self`). In Snippet B the function `external_greet` is defined outside the class and then assigned to the class attribute `greet`. Because it is a function object stored as a class attribute, attribute lookup on an instance (`b.greet`) also produces a bound method that passes the instance as `self`, so calling `b.greet()` behaves identically to `a.greet()`. Both approaches therefore produce the same runtime result.
-\nThe key differences lie in style and readability. Defining the method inside the class (Snippet A) follows the conventional, self‑documenting pattern that most Python programmers expect; the name `self` is merely a convention, but using it inside the class makes the code clearer. Assigning an external function (Snippet B) works technically, as the context notes, but it can confuse readers because the method’s implementation is not visually co‑located with the class definition, and the practice may be mistaken for a static function rather than an instance method. Moreover, the naming convention of the first parameter as `self` remains important for readability, even though Python does not enforce it. Thus, while both snippets bind correctly, Snippet A is generally preferred for maintainability and to avoid the pitfalls of hidden method definitions highlighted in the context.</t>
+The key differences lie in style and readability. Defining the method inside the class (Snippet A) follows the conventional, self‑documenting pattern that most Python programmers expect; the name `self` is merely a convention, but using it inside the class makes the code clearer. Assigning an external function (Snippet B) works technically, as the context notes, but it can confuse readers because the method’s implementation is not visually co‑located with the class definition, and the practice may be mistaken for a static function rather than an instance method. Moreover, the naming convention of the first parameter as `self` remains important for readability, even though Python does not enforce it. Thus, while both snippets bind correctly, Snippet A is generally preferred for maintainability and to avoid the pitfalls of hidden method definitions highlighted in the context.</t>
         </is>
       </c>
       <c r="M104" s="4" t="inlineStr">
@@ -10151,9 +10202,13 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="P104" s="4" t="n"/>
-    </row>
-    <row r="105" customFormat="1" s="8">
+      <c r="P104" s="4" t="inlineStr">
+        <is>
+          <t>AUDIT: validate_benchmark.py deep-check (2026-08). Generated_Question and Reference_Answer contained literal backslash-n escape sequences instead of real line breaks, making the code blocks unusable as shown. Content/reasoning was correct -- replaced literal \\n with real newlines in both fields, no wording changed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="183" customFormat="1" customHeight="1" s="8">
       <c r="A105" s="7" t="inlineStr">
         <is>
           <t>T7_017</t>
@@ -10201,267 +10256,4458 @@
       </c>
       <c r="J105" s="7" t="inlineStr">
         <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K105" s="4" t="inlineStr">
+        <is>
+          <t>Consider the following Python code that demonstrates inheritance and method overriding:
+```python
+class Vehicle:
+    def start(self):
+        print("Engine started")
+class Car(Vehicle):
+    def start(self):
+        # Overridden without calling the base implementation
+        print("Car is ready to go")
+```
+Evaluate the design of the `Car.start` method with respect to best‑practice principles for overriding methods in a subclass. Is the current implementation appropriate if the intention is to *extend* the behavior of `Vehicle.start`? Propose a concrete change to the code that follows best practice, and explain why your change improves the design.</t>
+        </is>
+      </c>
+      <c r="L105" s="4" t="inlineStr">
+        <is>
+          <t>The current `Car.start` method completely replaces the base implementation, discarding the useful side‑effect of printing "Engine started". When a subclass intends to *extend* rather than replace a base‑class method, best practice is to invoke the base method (typically via `super()`) and then add the subclass‑specific behavior. This preserves the contract of the base class and avoids code duplication if the base implementation changes later. A corrected version would be:
+```python
+class Car(Vehicle):
+    def start(self):
+        super().start()          # call the base class implementation
+        print("Car is ready to go")
+```
+By calling `super().start()` the `Car` class retains the original engine‑starting message while still providing its own additional output, resulting in clearer, more maintainable code that respects inheritance principles.</t>
+        </is>
+      </c>
+      <c r="M105" s="4" t="inlineStr">
+        <is>
+          <t>topic_7_oop.pdf_38, topic_7_oop.pdf_39, topic_7_oop.pdf_40, topic_7_oop.pdf_41</t>
+        </is>
+      </c>
+      <c r="N105" s="4" t="inlineStr">
+        <is>
+          <t>Calling super in overridden methods</t>
+        </is>
+      </c>
+      <c r="O105" s="7" t="inlineStr">
+        <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="K105" s="4" t="n"/>
-      <c r="L105" s="4" t="n"/>
-      <c r="M105" s="4" t="n"/>
-      <c r="N105" s="4" t="n"/>
-      <c r="O105" s="7" t="inlineStr">
+      <c r="P105" s="4" t="n"/>
+    </row>
+    <row r="106" ht="320" customFormat="1" customHeight="1" s="8">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>T7_018</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr">
+        <is>
+          <t>T7</t>
+        </is>
+      </c>
+      <c r="C106" s="7" t="inlineStr">
+        <is>
+          <t>Object-Oriented Programming</t>
+        </is>
+      </c>
+      <c r="D106" s="7" t="inlineStr">
+        <is>
+          <t>topic_7_oop.pdf</t>
+        </is>
+      </c>
+      <c r="E106" s="7" t="inlineStr">
+        <is>
+          <t>Evaluate</t>
+        </is>
+      </c>
+      <c r="F106" s="7" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G106" s="7" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="H106" s="7" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="I106" s="7" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J106" s="7" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K106" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Consider the following Python code that follows the pattern described in the context:
+```python
+class Mapping:
+    def __init__(self, iterable):
+        self.items_list = []
+        self.__update(iterable)
+    def update(self, iterable):
+        for item in iterable:
+            self.items_list.append(item)
+    __update = update   # private copy of original update()
+class MappingSubclass(Mapping):
+    def update(self, keys, values):
+        # new signature, does not call super().update()
+        for item in zip(keys, values):
+            self.items_list.append(item)
+    def __helper(self, data):
+        # attempt to reuse the private update logic from Mapping
+        self.__update(data)
+```
+A developer claims that calling `MappingSubclass(['a', 'b'])._MappingSubclass__helper(['c', 'd'])` will correctly add the elements `'c'` and `'d'` to `items_list` by re‑using the private `__update` method defined in `Mapping`. Evaluate this claim: does the call work as intended? If not, identify exactly why it fails according to Python’s name‑mangling rules and describe how the code should be modified so that `MappingSubclass` can safely invoke the original private update logic without breaking `__init__`.
+</t>
+        </is>
+      </c>
+      <c r="L106" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The claim is false. Inside `MappingSubclass`, the identifier `__update` is mangled to `_MappingSubclass__update`. Because `MappingSubclass` never defines a `__update` attribute, the lookup `self.__update` in `__helper` looks for `_MappingSubclass__update`, which does not exist, leading to an `AttributeError` and preventing the intended addition of `'c'` and `'d'`. The original private method created in `Mapping` was mangled to `_Mapping__update`, so `MappingSubclass` must reference that name explicitly (e.g., `self._Mapping__update(data)`) or use `super()` with the mangled name. A corrected version of `__helper` could be:
+```python
+    def __helper(self, data):
+        self._Mapping__update(data)   # call the private method from the base class
+```
+With this change, the call `MappingSubclass(['a', 'b'])._MappingSubclass__helper(['c', 'd'])` will correctly append `'c'` and `'d'` to `items_list` without breaking `__init__`.
+</t>
+        </is>
+      </c>
+      <c r="M106" s="4" t="inlineStr">
+        <is>
+          <t>topic_7_oop.pdf_48, topic_7_oop.pdf_49, topic_7_oop.pdf_50, topic_7_oop.pdf_51</t>
+        </is>
+      </c>
+      <c r="N106" s="4" t="inlineStr">
+        <is>
+          <t>Name Mangling Evaluation</t>
+        </is>
+      </c>
+      <c r="O106" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="P105" s="4" t="n"/>
-    </row>
-    <row r="106" customFormat="1" s="8">
-      <c r="A106" s="7" t="inlineStr">
-        <is>
-          <t>T7_018</t>
-        </is>
-      </c>
-      <c r="B106" s="7" t="inlineStr">
+      <c r="P106" s="4" t="n"/>
+    </row>
+    <row r="107" ht="57" customFormat="1" customHeight="1" s="8">
+      <c r="A107" s="7" t="inlineStr">
+        <is>
+          <t>T7_019</t>
+        </is>
+      </c>
+      <c r="B107" s="7" t="inlineStr">
         <is>
           <t>T7</t>
         </is>
       </c>
-      <c r="C106" s="7" t="inlineStr">
+      <c r="C107" s="7" t="inlineStr">
         <is>
           <t>Object-Oriented Programming</t>
         </is>
       </c>
-      <c r="D106" s="7" t="inlineStr">
+      <c r="D107" s="7" t="inlineStr">
         <is>
           <t>topic_7_oop.pdf</t>
         </is>
       </c>
-      <c r="E106" s="7" t="inlineStr">
+      <c r="E107" s="7" t="inlineStr">
         <is>
           <t>Evaluate</t>
         </is>
       </c>
-      <c r="F106" s="7" t="inlineStr">
+      <c r="F107" s="7" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
       </c>
-      <c r="G106" s="7" t="inlineStr">
+      <c r="G107" s="7" t="inlineStr">
         <is>
           <t>R4</t>
         </is>
       </c>
-      <c r="H106" s="7" t="inlineStr">
+      <c r="H107" s="7" t="inlineStr">
+        <is>
+          <t>Best Practice</t>
+        </is>
+      </c>
+      <c r="I107" s="7" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J107" s="7" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K107" s="4" t="inlineStr">
+        <is>
+          <t>Consider the following Python classes that use name‑mangling for a private copy of the original ``update`` method:
+```python
+class Mapping:
+    def __init__(self, iterable=None):
+        self.items_list = []
+        if iterable:
+            self.__update(iterable)
+    def update(self, iterable):
+        for item in iterable:
+            self.items_list.append(item)
+    __update = update  # private copy
+class MappingSubclass(Mapping):
+    def update(self, keys, values):
+        # new signature, does not call Mapping.__init__
+        for item in zip(keys, values):
+            self.items_list.append(item)
+    __update = update  # private copy in subclass
+```
+Evaluate the design from a best‑practice perspective. Does using double‑underscore ``__update`` and changing the method signature in the subclass adhere to good OOP principles in Python? Identify any problems and propose a more maintainable alternative implementation.</t>
+        </is>
+      </c>
+      <c r="L107" s="4" t="inlineStr">
+        <is>
+          <t>Using a double‑underscore name creates name‑mangling (e.g., ``_Mapping__update``) which hides the method from subclasses. While this prevents accidental overrides, it also makes intentional extension difficult, as the subclass cannot reliably call the original implementation without knowing the mangled name. Changing the signature of ``update`` in the subclass breaks the Liskov Substitution Principle: code that expects a Mapping instance to accept a single iterable will fail when passed a MappingSubclass. A better practice is to keep the public API stable—use a single‑underscore ``_update`` (protected) or keep the original ``update`` signature and accept flexible arguments (e.g., ``def update(self, *args, **kwargs)``). The subclass can then call ``super().update(...)`` with an appropriate iterable, preserving compatibility and avoiding name‑mangling pitfalls.</t>
+        </is>
+      </c>
+      <c r="M107" s="4" t="inlineStr">
+        <is>
+          <t>topic_7_oop.pdf_49, topic_7_oop.pdf_50, topic_7_oop.pdf_51, topic_7_oop.pdf_52</t>
+        </is>
+      </c>
+      <c r="N107" s="4" t="inlineStr">
+        <is>
+          <t>Name mangling and method overriding best practices</t>
+        </is>
+      </c>
+      <c r="O107" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P107" s="4" t="inlineStr">
+        <is>
+          <t>AUDIT: validate_benchmark.py deep-check (2026-08). Generated_Question contained literal backslash-n escape sequences instead of real line breaks, making the code blocks unusable as shown. Content/reasoning was correct -- replaced literal \\n with real newlines, no wording changed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="225" customFormat="1" customHeight="1" s="8">
+      <c r="A108" s="7" t="inlineStr">
+        <is>
+          <t>T7_020</t>
+        </is>
+      </c>
+      <c r="B108" s="7" t="inlineStr">
+        <is>
+          <t>T7</t>
+        </is>
+      </c>
+      <c r="C108" s="7" t="inlineStr">
+        <is>
+          <t>Object-Oriented Programming</t>
+        </is>
+      </c>
+      <c r="D108" s="7" t="inlineStr">
+        <is>
+          <t>topic_7_oop.pdf</t>
+        </is>
+      </c>
+      <c r="E108" s="7" t="inlineStr">
+        <is>
+          <t>Evaluate</t>
+        </is>
+      </c>
+      <c r="F108" s="7" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G108" s="7" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="H108" s="7" t="inlineStr">
+        <is>
+          <t>Best Practice</t>
+        </is>
+      </c>
+      <c r="I108" s="7" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J108" s="7" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K108" s="4" t="inlineStr">
+        <is>
+          <t>Consider the following class and two ways of using its method `greet`:
+```python
+class Greeter:
+    def greet(self):
+        return 'hello world'
+# Approach A
+g = Greeter()
+msg_func = g.greet  # stores the method object
+print(msg_func())
+# Approach B
+g = Greeter()
+print(g.greet())  # calls the method directly
+```
+Evaluate which approach follows best practice for invoking instance methods in Python. In your answer, discuss the implications of storing a method object versus calling the method directly, referring to how method binding works as described in the context.</t>
+        </is>
+      </c>
+      <c r="L108" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Approach B—calling the method directly with `g.greet()`—is the preferred practice in typical code.  When `g.greet` is accessed, Python creates a *method object* that binds the instance `g` to the underlying function `Greeter.greet`.  Storing that method object (as in Approach A) is legal and can be useful when the same bound method will be invoked many times or passed around, but it introduces an unnecessary intermediate object and can obscure the intent that the method is being called on the instance.  Directly calling `g.greet()` makes the binding implicit, is more readable, and avoids the tiny overhead of creating and later invoking a separate method object.  Therefore, unless there is a specific need to keep a reference to the bound method, the best‑practice recommendation is to call the method directly.
+</t>
+        </is>
+      </c>
+      <c r="M108" s="4" t="inlineStr">
+        <is>
+          <t>topic_7_oop.pdf_26, topic_7_oop.pdf_27, topic_7_oop.pdf_28, topic_7_oop.pdf_29</t>
+        </is>
+      </c>
+      <c r="N108" s="4" t="inlineStr">
+        <is>
+          <t>Method binding best practice</t>
+        </is>
+      </c>
+      <c r="O108" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P108" s="4" t="n"/>
+    </row>
+    <row r="109" ht="267" customFormat="1" customHeight="1" s="8">
+      <c r="A109" s="7" t="inlineStr">
+        <is>
+          <t>T7_021</t>
+        </is>
+      </c>
+      <c r="B109" s="7" t="inlineStr">
+        <is>
+          <t>T7</t>
+        </is>
+      </c>
+      <c r="C109" s="7" t="inlineStr">
+        <is>
+          <t>Object-Oriented Programming</t>
+        </is>
+      </c>
+      <c r="D109" s="7" t="inlineStr">
+        <is>
+          <t>topic_7_oop.pdf</t>
+        </is>
+      </c>
+      <c r="E109" s="7" t="inlineStr">
+        <is>
+          <t>Evaluate</t>
+        </is>
+      </c>
+      <c r="F109" s="7" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G109" s="7" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="H109" s="7" t="inlineStr">
         <is>
           <t>Scenario</t>
         </is>
       </c>
-      <c r="I106" s="7" t="inlineStr">
+      <c r="I109" s="7" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
       </c>
-      <c r="J106" s="7" t="inlineStr">
+      <c r="J109" s="7" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K109" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Consider the following Python classes that illustrate multiple inheritance and method overriding:
+```python
+class BaseA:
+    def process(self):
+        return "BaseA"
+class BaseB:
+    def process(self):
+        return "BaseB"
+class Derived(BaseA, BaseB):
+    def process(self):
+        # Attempt to extend the base implementation
+        result = BaseA.process(self) + "+Derived"
+        return result
+```
+A client creates an instance `d = Derived()` and calls `d.process()`. Evaluate whether the `process` method in `Derived` correctly extends the intended base class method according to Python’s inheritance rules described in the context. Identify which base class method is actually invoked, explain why, and state what change (if any) should be made to achieve the intended behavior of extending the method from the first base class in the inheritance list.
+</t>
+        </is>
+      </c>
+      <c r="L109" s="4" t="inlineStr">
+        <is>
+          <t>When `d.process()` is called, Python follows the method‑resolution order (MRO) for `Derived`, which is depth‑first, left‑to‑right: `Derived → BaseA → BaseB → object`. The overridden `process` in `Derived` explicitly calls `BaseA.process(self)`, so the method from `BaseA` is invoked, returning "BaseA". The result becomes "BaseA+Derived", which matches the intention of extending the first base class (`BaseA`). Therefore, the code already calls the intended base method; no change is required. If the intention had been to extend the next method in the MRO (i.e., `BaseB.process`), the call should use `super().process()` instead of `BaseA.process(self)`.</t>
+        </is>
+      </c>
+      <c r="M109" s="4" t="inlineStr">
+        <is>
+          <t>topic_7_oop.pdf_40, topic_7_oop.pdf_41, topic_7_oop.pdf_42, topic_7_oop.pdf_43</t>
+        </is>
+      </c>
+      <c r="N109" s="4" t="inlineStr">
+        <is>
+          <t>Method Resolution Order Evaluation</t>
+        </is>
+      </c>
+      <c r="O109" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="K106" s="4" t="n"/>
-      <c r="L106" s="4" t="n"/>
-      <c r="M106" s="4" t="n"/>
-      <c r="N106" s="4" t="n"/>
-      <c r="O106" s="7" t="inlineStr">
+      <c r="P109" s="4" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="9" t="inlineStr">
+        <is>
+          <t>T1_012</t>
+        </is>
+      </c>
+      <c r="B110" s="9" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="C110" s="9" t="inlineStr">
+        <is>
+          <t>Python Introduction &amp; Basics</t>
+        </is>
+      </c>
+      <c r="D110" s="9" t="inlineStr">
+        <is>
+          <t>topic_1_basics.pdf</t>
+        </is>
+      </c>
+      <c r="E110" s="9" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="F110" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G110" s="9" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="H110" s="9" t="inlineStr">
+        <is>
+          <t>Enumeration</t>
+        </is>
+      </c>
+      <c r="I110" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J110" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K110" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following Python code snippet:
+```python
+s1 = 'First line.\nSecond line.'
+s2 = r'C:\this\name'
+s3 = """\
+Usage: thingy [OPTIONS]
+-h Display this usage message
+"""
+```
+Based solely on the context provided, enumerate each distinct type of string literal demonstrated (s1, s2, s3) and briefly state how each type handles escape sequences or initial newlines.</t>
+        </is>
+      </c>
+      <c r="L110" s="9" t="inlineStr">
+        <is>
+          <t>1) **Regular string** (`s1`): Uses ordinary quotes. Escape sequences like `\n` are interpreted, so `\n` becomes an actual newline when the string is printed.
+2) **Raw string** (`s2`): Prefixed with `r`. Backslashes are treated literally; escape sequences are **not** processed, so the path is printed exactly as `C:\this\name`.
+3) **Triple‑quoted string with a leading backslash** (`s3`): Enclosed in triple quotes, allowing the string to span multiple lines. The leading backslash (`\`) on the first line suppresses the initial newline that would otherwise be included, while the remaining line breaks are preserved in the string.</t>
+        </is>
+      </c>
+      <c r="M110" s="9" t="inlineStr">
+        <is>
+          <t>topic_1_basics.pdf_9, topic_1_basics.pdf_10, topic_1_basics.pdf_11</t>
+        </is>
+      </c>
+      <c r="N110" s="9" t="inlineStr">
+        <is>
+          <t>String literal forms and newline handling</t>
+        </is>
+      </c>
+      <c r="O110" s="9" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="P106" s="4" t="n"/>
-    </row>
-    <row r="107" customFormat="1" s="8">
-      <c r="A107" s="7" t="inlineStr">
-        <is>
-          <t>T7_019</t>
-        </is>
-      </c>
-      <c r="B107" s="7" t="inlineStr">
+      <c r="P110" s="9" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="9" t="inlineStr">
+        <is>
+          <t>T1_013</t>
+        </is>
+      </c>
+      <c r="B111" s="9" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="C111" s="9" t="inlineStr">
+        <is>
+          <t>Python Introduction &amp; Basics</t>
+        </is>
+      </c>
+      <c r="D111" s="9" t="inlineStr">
+        <is>
+          <t>topic_1_basics.pdf</t>
+        </is>
+      </c>
+      <c r="E111" s="9" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="F111" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G111" s="9" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="H111" s="9" t="inlineStr">
+        <is>
+          <t>Enumeration</t>
+        </is>
+      </c>
+      <c r="I111" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J111" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K111" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following interactive Python session:
+```python
+&gt;&gt;&gt; tax = 12.5 / 100
+&gt;&gt;&gt; price = 100.50
+&gt;&gt;&gt; price * tax
+&gt;&gt;&gt; price + _
+&gt;&gt;&gt; round(_, 2)
+```
+Based on the description of the special variable `_` in the context, list the value produced by each expression in the order shown (including the assignments).</t>
+        </is>
+      </c>
+      <c r="L111" s="9" t="inlineStr">
+        <is>
+          <t>- `tax = 12.5 / 100` evaluates to **0.125**
+- `price = 100.50` evaluates to **100.5**
+- `price * tax` evaluates to **12.5625**
+- `price + _` (where `_` holds the previous result 12.5625) evaluates to **113.0625**
+- `round(_, 2)` (where `_` now holds 113.0625) evaluates to **113.06**</t>
+        </is>
+      </c>
+      <c r="M111" s="9" t="inlineStr">
+        <is>
+          <t>topic_1_basics.pdf_6, topic_1_basics.pdf_7, topic_1_basics.pdf_8</t>
+        </is>
+      </c>
+      <c r="N111" s="9" t="inlineStr">
+        <is>
+          <t>Using the underscore (_) as a read‑only result placeholder</t>
+        </is>
+      </c>
+      <c r="O111" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P111" s="9" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="9" t="inlineStr">
+        <is>
+          <t>T1_014</t>
+        </is>
+      </c>
+      <c r="B112" s="9" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="C112" s="9" t="inlineStr">
+        <is>
+          <t>Python Introduction &amp; Basics</t>
+        </is>
+      </c>
+      <c r="D112" s="9" t="inlineStr">
+        <is>
+          <t>topic_1_basics.pdf</t>
+        </is>
+      </c>
+      <c r="E112" s="9" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="F112" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G112" s="9" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="H112" s="9" t="inlineStr">
+        <is>
+          <t>Enumeration</t>
+        </is>
+      </c>
+      <c r="I112" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J112" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K112" s="9" t="inlineStr">
+        <is>
+          <t>Consider the string `word = 'Python'`. Enumerate the result of each of the following expressions as described in the context:\n1. `word[-2:]`\n2. `word[:2] + word[2:]`\n3. `word[4:42]`\n4. `word[42:]`\n5. `word[42]`\nProvide the output or error for each item.</t>
+        </is>
+      </c>
+      <c r="L112" s="9" t="inlineStr">
+        <is>
+          <t>1. 'on' – the slice from the second‑last character to the end.\n2. 'Python' – concatenating the slice before index 2 with the slice from index 2 onward reproduces the original string.\n3. 'on' – slicing beyond the string length returns the characters up to the end without error.\n4. '' (empty string) – a slice starting at an out‑of‑range index returns an empty string.\n5. IndexError: string index out of range – using an out‑of‑range index (not a slice) raises an error.</t>
+        </is>
+      </c>
+      <c r="M112" s="9" t="inlineStr">
+        <is>
+          <t>topic_1_basics.pdf_16, topic_1_basics.pdf_17, topic_1_basics.pdf_18, topic_1_basics.pdf_19</t>
+        </is>
+      </c>
+      <c r="N112" s="9" t="inlineStr">
+        <is>
+          <t>String slicing behavior</t>
+        </is>
+      </c>
+      <c r="O112" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P112" s="9" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="9" t="inlineStr">
+        <is>
+          <t>T1_015</t>
+        </is>
+      </c>
+      <c r="B113" s="9" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="C113" s="9" t="inlineStr">
+        <is>
+          <t>Python Introduction &amp; Basics</t>
+        </is>
+      </c>
+      <c r="D113" s="9" t="inlineStr">
+        <is>
+          <t>topic_1_basics.pdf</t>
+        </is>
+      </c>
+      <c r="E113" s="9" t="inlineStr">
+        <is>
+          <t>Evaluate</t>
+        </is>
+      </c>
+      <c r="F113" s="9" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G113" s="9" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H113" s="9" t="inlineStr">
+        <is>
+          <t>Best Practice</t>
+        </is>
+      </c>
+      <c r="I113" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J113" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K113" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following Python snippet that prints Fibonacci numbers less than 1000:
+```python
+a, b = 0, 1
+while a &lt; 1000:
+    print(a, end=',')
+    a, b = b, a+b
+```
+Evaluate this code against Python best‑practice guidelines for readability, output formatting, and loop design. Identify any shortcomings and rewrite the snippet so that it follows best practices while producing the same sequence of numbers (without a trailing comma).</t>
+        </is>
+      </c>
+      <c r="L113" s="9" t="inlineStr">
+        <is>
+          <t>The original code works but violates several best‑practice conventions: (1) the variable names ``a`` and ``b`` are non‑descriptive; (2) using ``print(..., end=',')`` leaves a trailing comma after the last number and provides no spacing, making the output harder to read; (3) the loop mixes computation and output, which reduces clarity. A more idiomatic version defines a function, uses meaningful names, collects the numbers in a list, and prints them with ``', '.join`` to avoid a trailing delimiter:
+```python
+def fibonacci(limit: int) -&gt; list[int]:
+    """Return a list of Fibonacci numbers less than *limit*."""
+    numbers = []
+    prev, cur = 0, 1
+    while prev &lt; limit:
+        numbers.append(prev)
+        prev, cur = cur, prev + cur
+    return numbers
+print(', '.join(str(n) for n in fibonacci(1000)))
+```
+This version improves readability, produces the same numeric sequence, and formats the output without an extra comma at the end.</t>
+        </is>
+      </c>
+      <c r="M113" s="9" t="inlineStr">
+        <is>
+          <t>topic_1_basics.pdf_30</t>
+        </is>
+      </c>
+      <c r="N113" s="9" t="inlineStr">
+        <is>
+          <t>Print function best practices</t>
+        </is>
+      </c>
+      <c r="O113" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P113" s="9" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="9" t="inlineStr">
+        <is>
+          <t>T1_016</t>
+        </is>
+      </c>
+      <c r="B114" s="9" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="C114" s="9" t="inlineStr">
+        <is>
+          <t>Python Introduction &amp; Basics</t>
+        </is>
+      </c>
+      <c r="D114" s="9" t="inlineStr">
+        <is>
+          <t>topic_1_basics.pdf</t>
+        </is>
+      </c>
+      <c r="E114" s="9" t="inlineStr">
+        <is>
+          <t>Evaluate</t>
+        </is>
+      </c>
+      <c r="F114" s="9" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G114" s="9" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="H114" s="9" t="inlineStr">
+        <is>
+          <t>Best Practice</t>
+        </is>
+      </c>
+      <c r="I114" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J114" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K114" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Consider the following two Python programs that aim to print all Fibonacci numbers less than 1000. Both produce the same visible output, but they differ in how they use the `print` function and variable assignment.
+Program A (uses string concatenation and explicit newline handling):
+```python
+a, b = 0, 1
+while a &lt; 1000:
+    print(str(a) + ',')  # prints a comma after each number and forces a newline
+    a, b = b, a + b
+```
+Program B (uses `print` with the `end` argument and tuple unpacking):
+```python
+a, b = 0, 1
+while a &lt; 1000:
+    print(a, end=',')
+    a, b = b, a + b
+```
+**Question:** Evaluate which program follows best practice for printing a sequence in Python. In your answer, discuss readability, efficiency, and proper use of the `print` function as described in the context.
+</t>
+        </is>
+      </c>
+      <c r="L114" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Program B follows best practice. It leverages `print`’s ability to accept multiple arguments and the `end` parameter to place a comma after each value without inserting an extra newline, exactly as the context describes. This avoids the unnecessary conversion of the integer to a string and the explicit concatenation performed in Program A, making the code more readable and slightly more efficient. Additionally, both programs use tuple unpacking (`a, b = b, a + b`), which is idiomatic Python for swapping values, but Program B combines this with the proper `print` usage, resulting in cleaner, more Pythonic code.
+</t>
+        </is>
+      </c>
+      <c r="M114" s="9" t="inlineStr">
+        <is>
+          <t>topic_1_basics.pdf_30, topic_1_basics.pdf_31</t>
+        </is>
+      </c>
+      <c r="N114" s="9" t="inlineStr">
+        <is>
+          <t>Using print with end argument</t>
+        </is>
+      </c>
+      <c r="O114" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P114" s="9" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="9" t="inlineStr">
+        <is>
+          <t>T1_017</t>
+        </is>
+      </c>
+      <c r="B115" s="9" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="C115" s="9" t="inlineStr">
+        <is>
+          <t>Python Introduction &amp; Basics</t>
+        </is>
+      </c>
+      <c r="D115" s="9" t="inlineStr">
+        <is>
+          <t>topic_1_basics.pdf</t>
+        </is>
+      </c>
+      <c r="E115" s="9" t="inlineStr">
+        <is>
+          <t>Evaluate</t>
+        </is>
+      </c>
+      <c r="F115" s="9" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G115" s="9" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="H115" s="9" t="inlineStr">
+        <is>
+          <t>Best Practice</t>
+        </is>
+      </c>
+      <c r="I115" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J115" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K115" s="9" t="inlineStr">
+        <is>
+          <t>The following code attempts to create a list of RGB colors and then extend it with an alpha channel. Evaluate whether the current approach follows best practices for handling mutable list objects. Identify any potential bugs related to list aliasing, and rewrite the code using a best‑practice method to avoid unintended side effects.
+```python
+rgb = ["Red", "Green", "Blue"]
+rgba = rgb
+rgba.append("Alpha")
+print("rgb:", rgb)
+print("rgba:", rgba)
+```</t>
+        </is>
+      </c>
+      <c r="L115" s="9" t="inlineStr">
+        <is>
+          <t>The code creates an alias: `rgba = rgb` makes both variables reference the same list. Consequently, appending "Alpha" to `rgba` also mutates `rgb`, which is usually unintended and can cause bugs when the original RGB list is needed elsewhere. A best‑practice approach is to create an explicit shallow copy before modifying the new list. For example:
+```python
+rgb = ["Red", "Green", "Blue"]
+rgba = rgb[:]          # or rgb.copy() / list(rgb)
+rgba.append("Alpha")
+print("rgb:", rgb)   # ['Red', 'Green', 'Blue']
+print("rgba:", rgba) # ['Red', 'Green', 'Blue', 'Alpha']
+```
+Using a copy isolates the two lists, preserving the original `rgb` while allowing `rgba` to be extended safely.</t>
+        </is>
+      </c>
+      <c r="M115" s="9" t="inlineStr">
+        <is>
+          <t>topic_1_basics.pdf_21, topic_1_basics.pdf_22, topic_1_basics.pdf_23</t>
+        </is>
+      </c>
+      <c r="N115" s="9" t="inlineStr">
+        <is>
+          <t>List aliasing and copying</t>
+        </is>
+      </c>
+      <c r="O115" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P115" s="9" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="9" t="inlineStr">
+        <is>
+          <t>T2_020</t>
+        </is>
+      </c>
+      <c r="B116" s="9" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="C116" s="9" t="inlineStr">
+        <is>
+          <t>Control Flow &amp; Functions</t>
+        </is>
+      </c>
+      <c r="D116" s="9" t="inlineStr">
+        <is>
+          <t>topic_2_control_flow_and_functions.pdf</t>
+        </is>
+      </c>
+      <c r="E116" s="9" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="F116" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G116" s="9" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="H116" s="9" t="inlineStr">
+        <is>
+          <t>Enumeration</t>
+        </is>
+      </c>
+      <c r="I116" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J116" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K116" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following Python code snippets taken from the context:
+```python
+# Strategy: Iterate over a copy
+for user, status in users.copy().items():
+    if status == 'inactive':
+        del users[user]
+# Strategy: Create a new collection
+active_users = {}
+for user, status in users.items():
+    if status == 'active':
+        active_users[user] = status
+```
+Based on these snippets, enumerate the two distinct strategies presented for safely modifying a collection while iterating over it.</t>
+        </is>
+      </c>
+      <c r="L116" s="9" t="inlineStr">
+        <is>
+          <t>1. Iterate over a copy of the collection (e.g., using `users.copy().items()`) and modify the original collection inside the loop.
+2. Create a new collection (e.g., `active_users`) and populate it with the desired items while iterating over the original collection.</t>
+        </is>
+      </c>
+      <c r="M116" s="9" t="inlineStr">
+        <is>
+          <t>topic_2_control_flow_and_functions.pdf_2, topic_2_control_flow_and_functions.pdf_3, topic_2_control_flow_and_functions.pdf_4</t>
+        </is>
+      </c>
+      <c r="N116" s="9" t="inlineStr">
+        <is>
+          <t>Safe collection iteration</t>
+        </is>
+      </c>
+      <c r="O116" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P116" s="9" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="9" t="inlineStr">
+        <is>
+          <t>T2_021</t>
+        </is>
+      </c>
+      <c r="B117" s="9" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="C117" s="9" t="inlineStr">
+        <is>
+          <t>Control Flow &amp; Functions</t>
+        </is>
+      </c>
+      <c r="D117" s="9" t="inlineStr">
+        <is>
+          <t>topic_2_control_flow_and_functions.pdf</t>
+        </is>
+      </c>
+      <c r="E117" s="9" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="F117" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G117" s="9" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="H117" s="9" t="inlineStr">
+        <is>
+          <t>Enumeration</t>
+        </is>
+      </c>
+      <c r="I117" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J117" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K117" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following function definition:
+```python
+def combined_example(pos_only, /, standard, *, kwd_only):
+    print(pos_only, standard, kwd_only)
+```
+Enumerate each parameter of `combined_example` and state whether it is a positional‑only, positional‑or‑keyword, or keyword‑only argument.</t>
+        </is>
+      </c>
+      <c r="L117" s="9" t="inlineStr">
+        <is>
+          <t>- `pos_only` – positional‑only (appears before the `/` marker)
+- `standard` – positional‑or‑keyword (appears after `/` and before `*`)
+- `kwd_only` – keyword‑only (appears after the `*` marker)</t>
+        </is>
+      </c>
+      <c r="M117" s="9" t="inlineStr">
+        <is>
+          <t>topic_2_control_flow_and_functions.pdf_41, topic_2_control_flow_and_functions.pdf_42, topic_2_control_flow_and_functions.pdf_43, topic_2_control_flow_and_functions.pdf_44</t>
+        </is>
+      </c>
+      <c r="N117" s="9" t="inlineStr">
+        <is>
+          <t>Function parameter classification</t>
+        </is>
+      </c>
+      <c r="O117" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P117" s="9" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="9" t="inlineStr">
+        <is>
+          <t>T2_022</t>
+        </is>
+      </c>
+      <c r="B118" s="9" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="C118" s="9" t="inlineStr">
+        <is>
+          <t>Control Flow &amp; Functions</t>
+        </is>
+      </c>
+      <c r="D118" s="9" t="inlineStr">
+        <is>
+          <t>topic_2_control_flow_and_functions.pdf</t>
+        </is>
+      </c>
+      <c r="E118" s="9" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="F118" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G118" s="9" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="H118" s="9" t="inlineStr">
+        <is>
+          <t>Enumeration</t>
+        </is>
+      </c>
+      <c r="I118" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J118" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K118" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following Python code snippets that deal with a dictionary of users and their status:
+```python
+# Strategy 1: Iterate over a copy and delete inactive users
+users = {'Hans': 'active', 'Éléonore': 'inactive', ' ': 'active'}
+for user, status in users.copy().items():
+    if status == 'inactive':
+        del users[user]
+# Strategy 2: Create a new collection of only active users
+users = {'Hans': 'active', 'Éléonore': 'inactive', ' ': 'active'}
+active_users = {}
+for user, status in users.items():
+    if status == 'active':
+        active_users[user] = status
+```
+Based on the code above, **enumerate the two distinct strategies** presented for handling inactive users in the `users` dictionary.</t>
+        </is>
+      </c>
+      <c r="L118" s="9" t="inlineStr">
+        <is>
+          <t>1. **Iterate over a copy of the dictionary and delete entries whose status is `'inactive'`.** This avoids modifying the dictionary while iterating over it.
+2. **Create a new dictionary (`active_users`) and copy only the entries whose status is `'active'`.** The original dictionary remains unchanged, and the new collection contains only active users.</t>
+        </is>
+      </c>
+      <c r="M118" s="9" t="inlineStr">
+        <is>
+          <t>topic_2_control_flow_and_functions.pdf_3, topic_2_control_flow_and_functions.pdf_4, topic_2_control_flow_and_functions.pdf_5, topic_2_control_flow_and_functions.pdf_6</t>
+        </is>
+      </c>
+      <c r="N118" s="9" t="inlineStr">
+        <is>
+          <t>Dictionary iteration strategies</t>
+        </is>
+      </c>
+      <c r="O118" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P118" s="9" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="9" t="inlineStr">
+        <is>
+          <t>T2_023</t>
+        </is>
+      </c>
+      <c r="B119" s="9" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="C119" s="9" t="inlineStr">
+        <is>
+          <t>Control Flow &amp; Functions</t>
+        </is>
+      </c>
+      <c r="D119" s="9" t="inlineStr">
+        <is>
+          <t>topic_2_control_flow_and_functions.pdf</t>
+        </is>
+      </c>
+      <c r="E119" s="9" t="inlineStr">
+        <is>
+          <t>Evaluate</t>
+        </is>
+      </c>
+      <c r="F119" s="9" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G119" s="9" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H119" s="9" t="inlineStr">
+        <is>
+          <t>Best Practice</t>
+        </is>
+      </c>
+      <c r="I119" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J119" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K119" s="9" t="inlineStr">
+        <is>
+          <t>Consider the two class definitions and the function below that compute the Manhattan distance between two points using structural pattern matching. Both classes represent a point with attributes x and y, but they differ in how they expose positional matching.
+```python
+# Version A
+class PointA:
+    __match_args__ = ("x", "y")
+    def __init__(self, x, y):
+        self.x = x
+        self.y = y
+# Version B
+class PointB:
+    def __init__(self, x, y):
+        self.x = x
+        self.y = y
+```
+```python
+def manhattan(p1, p2):
+    match p1, p2:
+        case (PointA(x1, y1), PointA(x2, y2)):
+            return abs(x1 - x2) + abs(y1 - y2)
+        case (PointB(x=x1, y=y1), PointB(x=x2, y=y2)):
+            return abs(x1 - x2) + abs(y1 - y2)
+        case _:
+            raise TypeError("Unsupported point types")
+```
+Which class definition and corresponding pattern usage represents the best practice for leveraging positional parameters and `__match_args__` in pattern matching, and why? Evaluate the trade‑offs in readability, maintainability, and future extensibility.</t>
+        </is>
+      </c>
+      <c r="L119" s="9" t="inlineStr">
+        <is>
+          <t>Version A together with the positional pattern `(PointA(x1, y1), PointA(x2, y2))` is the better practice. By defining `__match_args__ = ("x", "y")`, the class explicitly documents the order in which its attributes should be matched, allowing concise positional patterns that read like a tuple of values. This makes the `match` clause shorter, avoids repetition of attribute names, and ensures that if the internal attribute names change but the logical ordering stays the same, the pattern still works without modification. In contrast, Version B relies on keyword patterns, which are more verbose and tie the pattern directly to the attribute names; any rename of `x` or `y` would require updating every pattern. Positional matching also aligns with the recommended way of handling dataclasses and other builtin classes that provide an ordering for their fields, improving readability and future extensibility.</t>
+        </is>
+      </c>
+      <c r="M119" s="9" t="inlineStr">
+        <is>
+          <t>topic_2_control_flow_and_functions.pdf_18</t>
+        </is>
+      </c>
+      <c r="N119" s="9" t="inlineStr">
+        <is>
+          <t>Structural Pattern Matching Best Practice</t>
+        </is>
+      </c>
+      <c r="O119" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P119" s="9" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="9" t="inlineStr">
+        <is>
+          <t>T2_024</t>
+        </is>
+      </c>
+      <c r="B120" s="9" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="C120" s="9" t="inlineStr">
+        <is>
+          <t>Control Flow &amp; Functions</t>
+        </is>
+      </c>
+      <c r="D120" s="9" t="inlineStr">
+        <is>
+          <t>topic_2_control_flow_and_functions.pdf</t>
+        </is>
+      </c>
+      <c r="E120" s="9" t="inlineStr">
+        <is>
+          <t>Evaluate</t>
+        </is>
+      </c>
+      <c r="F120" s="9" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G120" s="9" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="H120" s="9" t="inlineStr">
+        <is>
+          <t>Best Practice</t>
+        </is>
+      </c>
+      <c r="I120" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J120" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K120" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The following Python function mixes control flow and arithmetic, but it does not follow the style recommendations described in the context. Evaluate the code against those best‑practice guidelines and rewrite it so that it complies with PEP 8. In your answer, list at least three specific style violations and provide a corrected version of the function.
+```python
+def process(data):
+ total=0
+ for i in range(len(data)):
+  if data[i]%2==0:
+   total+=data[i]
+  else:
+   total+=data[i]*2
+return total
+```
+</t>
+        </is>
+      </c>
+      <c r="L120" s="9" t="inlineStr">
+        <is>
+          <t>**Style violations**
+1. Indentation uses a single space (or inconsistent spacing) instead of the required 4‑space blocks.
+2. Operators and commas lack surrounding spaces (e.g., `total=0`, `data[i]%2==0`, `total+=data[i]`).
+3. The function has no docstring and there is no blank line separating it from surrounding code, which PEP 8 recommends for readability.
+4. The return statement is not indented to the function block.
+**Corrected version**
+```python
+def process(data):
+    """Return the sum of even numbers and twice the odd numbers in *data*.
+    """
+    total = 0
+    for i in range(len(data)):
+        if data[i] % 2 == 0:
+            total += data[i]
+        else:
+            total += data[i] * 2
+    return total
+```
+The revised code uses 4‑space indentation, inserts spaces around all operators and after commas, adds a concise docstring, and leaves a blank line before the function definition, thereby satisfying the best‑practice guidelines from the context.</t>
+        </is>
+      </c>
+      <c r="M120" s="9" t="inlineStr">
+        <is>
+          <t>topic_2_control_flow_and_functions.pdf_61, topic_2_control_flow_and_functions.pdf_62</t>
+        </is>
+      </c>
+      <c r="N120" s="9" t="inlineStr">
+        <is>
+          <t>PEP8 function style</t>
+        </is>
+      </c>
+      <c r="O120" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P120" s="9" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="9" t="inlineStr">
+        <is>
+          <t>T2_025</t>
+        </is>
+      </c>
+      <c r="B121" s="9" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="C121" s="9" t="inlineStr">
+        <is>
+          <t>Control Flow &amp; Functions</t>
+        </is>
+      </c>
+      <c r="D121" s="9" t="inlineStr">
+        <is>
+          <t>topic_2_control_flow_and_functions.pdf</t>
+        </is>
+      </c>
+      <c r="E121" s="9" t="inlineStr">
+        <is>
+          <t>Evaluate</t>
+        </is>
+      </c>
+      <c r="F121" s="9" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G121" s="9" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="H121" s="9" t="inlineStr">
+        <is>
+          <t>Best Practice</t>
+        </is>
+      </c>
+      <c r="I121" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J121" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K121" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following function that attempts to remove all negative numbers from a list while iterating over it:
+```python
+def clean(nums):
+    for n in nums:
+        if n &lt; 0:
+            nums.remove(n)
+    return nums
+```
+Is this implementation a good practice? Evaluate the potential issues that can arise from modifying the list during iteration and rewrite the function using a best‑practice approach that safely removes the negative values.</t>
+        </is>
+      </c>
+      <c r="L121" s="9" t="inlineStr">
+        <is>
+          <t>Modifying a list while iterating over it is unsafe because the iterator sees a changing sequence; elements can be skipped or cause unexpected IndexError. In the example, when a negative number is removed, the next element shifts left, so the loop’s internal index moves past it and the subsequent negative value may remain in the list. A best‑practice solution is to iterate over a copy of the list or to build a new list that contains only the desired items. For example:
+```python
+def clean(nums):
+    # iterate over a shallow copy so removal does not affect the loop
+    for n in nums[:]:
+        if n &lt; 0:
+            nums.remove(n)
+    return nums
+```
+or more idiomatically using a list comprehension:
+```python
+def clean(nums):
+    return [n for n in nums if n &gt;= 0]
+```
+Both approaches avoid mutating the list while it is being traversed, ensuring all negative numbers are removed reliably.</t>
+        </is>
+      </c>
+      <c r="M121" s="9" t="inlineStr">
+        <is>
+          <t>topic_2_control_flow_and_functions.pdf_0, topic_2_control_flow_and_functions.pdf_1, topic_2_control_flow_and_functions.pdf_2</t>
+        </is>
+      </c>
+      <c r="N121" s="9" t="inlineStr">
+        <is>
+          <t>Safe list modification</t>
+        </is>
+      </c>
+      <c r="O121" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P121" s="9" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="9" t="inlineStr">
+        <is>
+          <t>T3_020</t>
+        </is>
+      </c>
+      <c r="B122" s="9" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C122" s="9" t="inlineStr">
+        <is>
+          <t>Core Data Structures</t>
+        </is>
+      </c>
+      <c r="D122" s="9" t="inlineStr">
+        <is>
+          <t>topic_3_data_structures.pdf</t>
+        </is>
+      </c>
+      <c r="E122" s="9" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="F122" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G122" s="9" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="H122" s="9" t="inlineStr">
+        <is>
+          <t>Enumeration</t>
+        </is>
+      </c>
+      <c r="I122" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J122" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K122" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following Python code taken from the context:
+```python
+a = set('abracadabra')
+b = set('alacazam')
+print(a)          # unique letters in a
+print(a - b)      # letters in a but not in b
+print(a | b)      # letters in a or b or both
+print(a &amp; b)      # letters in both a and b
+print(a ^ b)      # letters in a or b but not both
+```
+Based on this code, enumerate the exact contents of the sets printed for `a`, `a - b`, `a | b`, `a &amp; b`, and `a ^ b`.</t>
+        </is>
+      </c>
+      <c r="L122" s="9" t="inlineStr">
+        <is>
+          <t>- `a` → {'a', 'r', 'b', 'c', 'd'}
+- `a - b` → {'r', 'd', 'b'}
+- `a | b` → {'a', 'c', 'r', 'd', 'b', 'm', 'z', 'l'}
+- `a &amp; b` → {'a', 'c'}
+- `a ^ b` → {'r', 'd', 'b', 'm', 'z', 'l'}</t>
+        </is>
+      </c>
+      <c r="M122" s="9" t="inlineStr">
+        <is>
+          <t>topic_3_data_structures.pdf_24, topic_3_data_structures.pdf_25, topic_3_data_structures.pdf_26</t>
+        </is>
+      </c>
+      <c r="N122" s="9" t="inlineStr">
+        <is>
+          <t>Set operations</t>
+        </is>
+      </c>
+      <c r="O122" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P122" s="9" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="9" t="inlineStr">
+        <is>
+          <t>T3_021</t>
+        </is>
+      </c>
+      <c r="B123" s="9" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C123" s="9" t="inlineStr">
+        <is>
+          <t>Core Data Structures</t>
+        </is>
+      </c>
+      <c r="D123" s="9" t="inlineStr">
+        <is>
+          <t>topic_3_data_structures.pdf</t>
+        </is>
+      </c>
+      <c r="E123" s="9" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="F123" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G123" s="9" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="H123" s="9" t="inlineStr">
+        <is>
+          <t>Enumeration</t>
+        </is>
+      </c>
+      <c r="I123" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J123" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K123" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following Python session:
+&gt;&gt;&gt; a = [1, 66.25, 333, 333, 1234.5]
+&gt;&gt;&gt; del a[0]
+&gt;&gt;&gt; a
+&gt;&gt;&gt; del a[2:4]
+&gt;&gt;&gt; a
+&gt;&gt;&gt; del a[:]
+&gt;&gt;&gt; a
+&gt;&gt;&gt; del a
+List the exact contents of the list ``a`` after each ``del`` statement (the three deletions that operate on the list) and state what occurs if you try to reference ``a`` after the final ``del a`` statement.</t>
+        </is>
+      </c>
+      <c r="L123" s="9" t="inlineStr">
+        <is>
+          <t>- After ``del a[0]`` the list is ``[66.25, 333, 333, 1234.5]``.
+- After ``del a[2:4]`` the list becomes ``[66.25, 333]``.
+- After ``del a[:]`` the list is ``[]`` (empty).
+- After ``del a`` the name ``a`` is removed from the current namespace; any subsequent reference to ``a`` raises a ``NameError`` because the variable no longer exists.</t>
+        </is>
+      </c>
+      <c r="M123" s="9" t="inlineStr">
+        <is>
+          <t>topic_3_data_structures.pdf_17, topic_3_data_structures.pdf_18, topic_3_data_structures.pdf_19, topic_3_data_structures.pdf_20</t>
+        </is>
+      </c>
+      <c r="N123" s="9" t="inlineStr">
+        <is>
+          <t>effects of del on lists</t>
+        </is>
+      </c>
+      <c r="O123" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P123" s="9" t="inlineStr">
+        <is>
+          <t>AUDIT (2026-08): regenerated row still had wrong values -- 'after del a[0]' repeated the original unmodified list instead of applying the deletion, and 'after del a[2:4]' inherited that error. Verified correct sequence by direct execution: del a[0] -&gt; [66.25, 333, 333, 1234.5]; del a[2:4] -&gt; [66.25, 333]; del a[:] -&gt; []; del a then referencing a raises NameError (these last two were already correct). Reference_Answer corrected accordingly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="9" t="inlineStr">
+        <is>
+          <t>T3_022</t>
+        </is>
+      </c>
+      <c r="B124" s="9" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C124" s="9" t="inlineStr">
+        <is>
+          <t>Core Data Structures</t>
+        </is>
+      </c>
+      <c r="D124" s="9" t="inlineStr">
+        <is>
+          <t>topic_3_data_structures.pdf</t>
+        </is>
+      </c>
+      <c r="E124" s="9" t="inlineStr">
+        <is>
+          <t>Evaluate</t>
+        </is>
+      </c>
+      <c r="F124" s="9" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G124" s="9" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H124" s="9" t="inlineStr">
+        <is>
+          <t>Best Practice</t>
+        </is>
+      </c>
+      <c r="I124" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J124" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K124" s="9" t="inlineStr">
+        <is>
+          <t>Consider the two snippets below that generate a list of (x, y) pairs where x is taken from [1,2,3] and y from [3,1,4] only if x != y:
+Snippet A (list comprehension):
+```python
+pairs = [(x, y) for x in [1,2,3] for y in [3,1,4] if x != y]
+```
+Snippet B (explicit loops):
+```python
+pairs = []
+for x in [1,2,3]:
+    for y in [3,1,4]:
+        if x != y:
+            pairs.append((x, y))
+```
+Evaluate which snippet represents best practice for this specific task. Justify your choice by discussing readability, execution efficiency, and memory usage, and describe a scenario where the other approach would be preferable.</t>
+        </is>
+      </c>
+      <c r="L124" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The list‑comprehension version (Snippet A) is the best practice here because the operation is a simple, single‑line transformation with a clear filtering condition. It expresses the intent compactly, is idiomatic Python, and the underlying implementation is essentially the same as the nested loops, so there is no measurable performance penalty. Because it builds the full list in memory, it uses the same amount of memory as the loop version, but the readability gain outweighs that cost for a modest data size.
+The explicit‑loop version (Snippet B) would be preferable if the body of the loop became more complex—e.g., multiple statements, error handling, or intermediate calculations—where a list comprehension would become hard to read. Additionally, if the result were needed lazily rather than all at once, a generator expression would be a better choice than either snippet.
+</t>
+        </is>
+      </c>
+      <c r="M124" s="9" t="inlineStr">
+        <is>
+          <t>topic_3_data_structures.pdf_10</t>
+        </is>
+      </c>
+      <c r="N124" s="9" t="inlineStr">
+        <is>
+          <t>List comprehension vs loop best practice</t>
+        </is>
+      </c>
+      <c r="O124" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P124" s="9" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="9" t="inlineStr">
+        <is>
+          <t>T3_023</t>
+        </is>
+      </c>
+      <c r="B125" s="9" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C125" s="9" t="inlineStr">
+        <is>
+          <t>Core Data Structures</t>
+        </is>
+      </c>
+      <c r="D125" s="9" t="inlineStr">
+        <is>
+          <t>topic_3_data_structures.pdf</t>
+        </is>
+      </c>
+      <c r="E125" s="9" t="inlineStr">
+        <is>
+          <t>Evaluate</t>
+        </is>
+      </c>
+      <c r="F125" s="9" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G125" s="9" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H125" s="9" t="inlineStr">
+        <is>
+          <t>Best Practice</t>
+        </is>
+      </c>
+      <c r="I125" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J125" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K125" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following two implementations that aim to retrieve the first non‑empty string from a list `candidates`.
+Implementation A (uses short‑circuit `or`):
+```python
+candidates = ['', 'Trondheim', 'Hammer Dance']
+first = candidates[0] or candidates[1] or candidates[2]
+print(first)
+```
+Implementation B (uses an explicit loop):
+```python
+candidates = ['', 'Trondheim', 'Hammer Dance']
+first = None
+for s in candidates:
+    if s:
+        first = s
+        break
+print(first)
+```
+Which implementation follows best practice for readability, efficiency, and correct handling of an arbitrary‑length iterable? If you think either snippet has a flaw, rewrite it using the most Pythonic approach and explain why your version is preferable.</t>
+        </is>
+      </c>
+      <c r="L125" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implementation A only works when the number of elements is known in advance; adding or removing items requires changing the code, which harms maintainability. Implementation B works for any length but is more verbose than necessary. The most Pythonic best‑practice solution is to use a generator expression with ``next`` so the short‑circuiting is explicit and the code handles an arbitrary iterable cleanly:
+```python
+candidates = ['', 'Trondheim', 'Hammer Dance']
+first = next((s for s in candidates if s), None)
+print(first)
+```
+This version is readable, efficient (stops at the first truthy value), and scales to any size without manual indexing or loop boilerplate.
+</t>
+        </is>
+      </c>
+      <c r="M125" s="9" t="inlineStr">
+        <is>
+          <t>topic_3_data_structures.pdf_37</t>
+        </is>
+      </c>
+      <c r="N125" s="9" t="inlineStr">
+        <is>
+          <t>Short‑circuit default selection</t>
+        </is>
+      </c>
+      <c r="O125" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P125" s="9" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="9" t="inlineStr">
+        <is>
+          <t>T3_024</t>
+        </is>
+      </c>
+      <c r="B126" s="9" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C126" s="9" t="inlineStr">
+        <is>
+          <t>Core Data Structures</t>
+        </is>
+      </c>
+      <c r="D126" s="9" t="inlineStr">
+        <is>
+          <t>topic_3_data_structures.pdf</t>
+        </is>
+      </c>
+      <c r="E126" s="9" t="inlineStr">
+        <is>
+          <t>Evaluate</t>
+        </is>
+      </c>
+      <c r="F126" s="9" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G126" s="9" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="H126" s="9" t="inlineStr">
+        <is>
+          <t>Best Practice</t>
+        </is>
+      </c>
+      <c r="I126" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J126" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K126" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following Python code that uses plain lists to implement a stack and a queue:
+```python
+# Stack implementation using a list
+stack = []
+for i in range(5):
+    stack.append(i)
+while stack:
+    print(stack.pop())
+# Queue implementation using a list
+queue = []
+for i in range(5):
+    queue.append(i)
+while queue:
+    print(queue.pop(0))
+```
+Evaluate the suitability of these two implementations for production code. Identify any performance or correctness concerns, and recommend a best‑practice alternative for each data structure, justifying your choices with respect to time‑complexity and Python’s design principles for mutable sequences.</t>
+        </is>
+      </c>
+      <c r="L126" s="9" t="inlineStr">
+        <is>
+          <t>The stack implementation is appropriate: using ``list.append`` to push and ``list.pop()`` to retrieve the last element gives O(1) amortized time for both operations, matching the LIFO semantics described in the documentation. No correctness issues arise because ``pop()`` without an index always removes the most recently added item.
+The queue implementation is problematic. ``list.pop(0)`` removes the first element, which requires shifting all remaining items one position to the left; this incurs O(n) time per dequeue operation. In a real‑world scenario with many enqueues/dequeues, the overall cost becomes quadratic. The best‑practice solution is to use ``collections.deque`` which provides O(1) ``append`` and ``popleft`` operations. A corrected version:
+```python
+from collections import deque
+# Stack (still fine with list)
+stack = []
+for i in range(5):
+    stack.append(i)
+while stack:
+    print(stack.pop())
+# Queue using deque
+queue = deque()
+for i in range(5):
+    queue.append(i)
+while queue:
+    print(queue.popleft())
+```
+This respects Python’s design principle that mutable sequence methods modify in place and return ``None`` while delivering optimal performance for both LIFO and FIFO use cases.</t>
+        </is>
+      </c>
+      <c r="M126" s="9" t="inlineStr">
+        <is>
+          <t>topic_3_data_structures.pdf_5, topic_3_data_structures.pdf_6</t>
+        </is>
+      </c>
+      <c r="N126" s="9" t="inlineStr">
+        <is>
+          <t>Stack vs queue best practice</t>
+        </is>
+      </c>
+      <c r="O126" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P126" s="9" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="9" t="inlineStr">
+        <is>
+          <t>T3_025</t>
+        </is>
+      </c>
+      <c r="B127" s="9" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C127" s="9" t="inlineStr">
+        <is>
+          <t>Core Data Structures</t>
+        </is>
+      </c>
+      <c r="D127" s="9" t="inlineStr">
+        <is>
+          <t>topic_3_data_structures.pdf</t>
+        </is>
+      </c>
+      <c r="E127" s="9" t="inlineStr">
+        <is>
+          <t>Evaluate</t>
+        </is>
+      </c>
+      <c r="F127" s="9" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G127" s="9" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="H127" s="9" t="inlineStr">
+        <is>
+          <t>Best Practice</t>
+        </is>
+      </c>
+      <c r="I127" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J127" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K127" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following two implementations of a FIFO queue that process the list of integers `[1, 2, 3, 4, 5]`. Implementation A uses a plain Python list, while Implementation B uses `collections.deque`.
+```python
+# Implementation A – list as a queue
+queue_a = []
+for i in [1, 2, 3, 4, 5]:
+    queue_a.append(i)          # enqueue
+while queue_a:
+    item = queue_a.pop(0)      # dequeue from front
+    print(item, end=' ')
+```
+```python
+# Implementation B – deque as a queue
+from collections import deque
+queue_b = deque()
+for i in [1, 2, 3, 4, 5]:
+    queue_b.append(i)          # enqueue
+while queue_b:
+    item = queue_b.popleft()   # dequeue from front
+    print(item, end=' ')
+```
+Evaluate which implementation follows best practice for a queue in Python. In your answer, discuss time‑complexity of the enqueue/dequeue operations, readability, and any design principles mentioned in the provided context about mutable data structures.</t>
+        </is>
+      </c>
+      <c r="L127" s="9" t="inlineStr">
+        <is>
+          <t>Implementation B (using `collections.deque`) follows best practice for a FIFO queue. With a list, `pop(0)` requires shifting all remaining elements, giving O(n) time per dequeue, whereas `deque.popleft()` removes the leftmost element in O(1) time, making the overall algorithm linear. Both approaches have O(1) enqueue (`append`), but the deque avoids the hidden performance penalty of the list. Readability is comparable; `deque` explicitly signals a double‑ended queue, aligning with the design principle that mutable structures should be used in ways that match their intended operations. The context notes that list methods that modify the structure return `None` and that lists are naturally suited for stack usage (LIFO) via `append`/`pop()`. For a queue (FIFO), the deque’s dedicated methods (`append`/`popleft`) are the idiomatic and efficient choice.</t>
+        </is>
+      </c>
+      <c r="M127" s="9" t="inlineStr">
+        <is>
+          <t>topic_3_data_structures.pdf_4, topic_3_data_structures.pdf_5, topic_3_data_structures.pdf_6</t>
+        </is>
+      </c>
+      <c r="N127" s="9" t="inlineStr">
+        <is>
+          <t>Queue implementation best practice</t>
+        </is>
+      </c>
+      <c r="O127" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P127" s="9" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="9" t="inlineStr">
+        <is>
+          <t>T4_013</t>
+        </is>
+      </c>
+      <c r="B128" s="9" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C128" s="9" t="inlineStr">
+        <is>
+          <t>Modules &amp; Packages</t>
+        </is>
+      </c>
+      <c r="D128" s="9" t="inlineStr">
+        <is>
+          <t>topic_4_modules.pdf</t>
+        </is>
+      </c>
+      <c r="E128" s="9" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="F128" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G128" s="9" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="H128" s="9" t="inlineStr">
+        <is>
+          <t>Enumeration</t>
+        </is>
+      </c>
+      <c r="I128" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J128" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K128" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following Python snippet:
+```python
+import sys
+print(sys.path)
+```
+When this script is executed, Python initializes the module search path as described in the context. Enumerate the first two entries that will appear in the printed list, in the order they appear.</t>
+        </is>
+      </c>
+      <c r="L128" s="9" t="inlineStr">
+        <is>
+          <t>1) The directory containing the script that is being run.
+2) The standard‑library directory path (the standard library path).</t>
+        </is>
+      </c>
+      <c r="M128" s="9" t="inlineStr">
+        <is>
+          <t>topic_4_modules.pdf_12, topic_4_modules.pdf_13, topic_4_modules.pdf_14</t>
+        </is>
+      </c>
+      <c r="N128" s="9" t="inlineStr">
+        <is>
+          <t>module search path initialization</t>
+        </is>
+      </c>
+      <c r="O128" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P128" s="9" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="9" t="inlineStr">
+        <is>
+          <t>T4_014</t>
+        </is>
+      </c>
+      <c r="B129" s="9" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C129" s="9" t="inlineStr">
+        <is>
+          <t>Modules &amp; Packages</t>
+        </is>
+      </c>
+      <c r="D129" s="9" t="inlineStr">
+        <is>
+          <t>topic_4_modules.pdf</t>
+        </is>
+      </c>
+      <c r="E129" s="9" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="F129" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G129" s="9" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="H129" s="9" t="inlineStr">
+        <is>
+          <t>Enumeration</t>
+        </is>
+      </c>
+      <c r="I129" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J129" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K129" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following Python snippet:
+```python
+import sys
+print(dir(sys))
+```
+Based solely on the provided context, enumerate all of the attribute names that the call to `dir(sys)` would include.</t>
+        </is>
+      </c>
+      <c r="L129" s="9" t="inlineStr">
+        <is>
+          <t>call_tracing, callstats, copyright, displayhook, dont_write_bytecode, exc_info, excepthook, exec_prefix, executable, exit, flags, float_info, float_repr_style, get_asyncgen_hooks, get_coroutine_origin_tracking_depth, getallocatedblocks, getdefaultencoding, getdlopenflags, getfilesystemencodeerrors, getfilesystemencoding, getprofile, getrecursionlimit, getrefcount, getsizeof, getswitchinterval, gettrace, hash_info, hexversion, implementation, int_info, intern, is_finalizing, last_traceback, last_type, last_value, maxsize, maxunicode, meta_path, modules, path, path_hooks, path_importer_cache, platform, prefix, ps1, ps2, pycache_prefix, set_asyncgen_hooks, set_coroutine_origin_tracking_depth, setdlopenflags, setprofile, setrecursionlimit, setswitchinterval, settrace, stderr, stdin, stdout, thread_info, unraisablehook, version, version_info, warnoptions</t>
+        </is>
+      </c>
+      <c r="M129" s="9" t="inlineStr">
+        <is>
+          <t>topic_4_modules.pdf_21, topic_4_modules.pdf_22, topic_4_modules.pdf_23, topic_4_modules.pdf_24</t>
+        </is>
+      </c>
+      <c r="N129" s="9" t="inlineStr">
+        <is>
+          <t>sys module attribute enumeration</t>
+        </is>
+      </c>
+      <c r="O129" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P129" s="9" t="n"/>
+    </row>
+    <row r="130" ht="160" customHeight="1">
+      <c r="A130" s="9" t="inlineStr">
+        <is>
+          <t>T4_015</t>
+        </is>
+      </c>
+      <c r="B130" s="9" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C130" s="9" t="inlineStr">
+        <is>
+          <t>Modules &amp; Packages</t>
+        </is>
+      </c>
+      <c r="D130" s="9" t="inlineStr">
+        <is>
+          <t>topic_4_modules.pdf</t>
+        </is>
+      </c>
+      <c r="E130" s="9" t="inlineStr">
+        <is>
+          <t>Evaluate</t>
+        </is>
+      </c>
+      <c r="F130" s="9" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G130" s="9" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H130" s="9" t="inlineStr">
+        <is>
+          <t>Best Practice</t>
+        </is>
+      </c>
+      <c r="I130" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J130" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K130" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Consider the following two files that are part of a package named **utils**. The package is used in a larger project that frequently calls ``dir()`` to inspect the current namespace.
+```python
+# utils/math_ops.py
+PI = 3.14159
+_epsilon = 1e-10
+def add(a, b):
+    return a + b
+def _private_helper(x):
+    return x * _epsilon
+# utils/__init__.py
+from .math_ops import *  # noqa: F403
+# main.py (client code)
+import utils
+from utils import *
+print(dir())
+```
+The code runs without error, but it mixes public and private symbols and relies on ``import *`` both inside the package and in client code. **Evaluate** the design of this module/package according to best‑practice principles. Identify **at least three** concrete issues, explain why each is problematic, and propose a specific change (e.g., modify an import line, add a variable, rename something) that would improve the package’s maintainability and namespace cleanliness.
+</t>
+        </is>
+      </c>
+      <c r="L130" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. **Wildcard import inside the package (`from .math_ops import *`), with no `__all__` defined.** Note: Python's `import *` automatically skips names starting with an underscore, so `_epsilon` and `_private_helper` are NOT actually pulled in here. The real problem is that without `__all__`, every non-underscore name in `math_ops` is exported implicitly -- including anything added later (e.g. a forgotten `import os` at module level, or a new helper that isn't underscore-prefixed) -- so the public surface is undocumented and can grow by accident. *Improvement:* add `__all__ = ['add', 'PI']` to `math_ops.py`, or replace the wildcard with explicit imports, e.g. ``from .math_ops import add, PI``.
+2. **Wildcard import in client code (`from utils import *`).** This adds all names from ``utils`` (including the private ones that leaked through the package) to the caller’s global namespace, defeating the purpose of encapsulation and making ``dir()`` noisy. *Improvement:* have client code import only what it needs, e.g. ``from utils import add, PI``.
+3. **Missing ``__all__`` declaration in ``utils/__init__.py``.** Without ``__all__`` the package cannot control which symbols are exported when ``import *`` is used, so private names are unintentionally exposed. Defining ``__all__ = ['add', 'PI']`` explicitly limits the public API and keeps ``dir()`` output tidy.
+Additional minor fix: rename ``_epsilon`` to a single leading underscore (already done) and keep it out of the exported list. Together, these changes keep the namespace clean, make the intended public interface obvious, and prevent accidental reliance on internal helpers.
+</t>
+        </is>
+      </c>
+      <c r="M130" s="9" t="inlineStr">
+        <is>
+          <t>topic_4_modules.pdf_22</t>
+        </is>
+      </c>
+      <c r="N130" s="9" t="inlineStr">
+        <is>
+          <t>Evaluating module namespace hygiene</t>
+        </is>
+      </c>
+      <c r="O130" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P130" s="9" t="inlineStr">
+        <is>
+          <t>AUDIT: validate_benchmark.py deep-check + manual verification (2026-08). Original violation #1 claimed `import *` pulls in `_epsilon`/`_private_helper`. Ran the actual package -- confirmed this is false (Python excludes underscore-prefixed names from wildcard imports by default). Violation #1 rewritten to state the real risk (undocumented public surface via missing __all__). Violations #2 and #3 were correct, unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="9" t="inlineStr">
+        <is>
+          <t>T4_016</t>
+        </is>
+      </c>
+      <c r="B131" s="9" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C131" s="9" t="inlineStr">
+        <is>
+          <t>Modules &amp; Packages</t>
+        </is>
+      </c>
+      <c r="D131" s="9" t="inlineStr">
+        <is>
+          <t>topic_4_modules.pdf</t>
+        </is>
+      </c>
+      <c r="E131" s="9" t="inlineStr">
+        <is>
+          <t>Evaluate</t>
+        </is>
+      </c>
+      <c r="F131" s="9" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G131" s="9" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="H131" s="9" t="inlineStr">
+        <is>
+          <t>Best Practice</t>
+        </is>
+      </c>
+      <c r="I131" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J131" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K131" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following Python script:
+```python
+import sys
+# Attempt to ensure our local version of 'spam' is imported
+sys.path.insert(0, '/opt/custom_lib')
+import spam
+```
+Assume there is a built‑in module named `spam` and also a file `/opt/custom_lib/spam.py` containing a local implementation. Evaluate the best‑practice approach for guaranteeing that the local `spam` module is imported, considering the import search order described in the context. In your answer, discuss the effectiveness of the shown code, any potential pitfalls, and propose a more robust solution that adheres to Python’s module import conventions.</t>
+        </is>
+      </c>
+      <c r="L131" s="9" t="inlineStr">
+        <is>
+          <t>The snippet tries to force the local `spam` by inserting its directory at the front of `sys.path`, but according to the context the interpreter always looks for a built‑in module **before** consulting any entries in `sys.path`. Therefore the code will still import the built‑in `spam` and the modification of `sys.path` has no effect on that search order. Moreover, changing `sys.path` at runtime is fragile: it only affects imports that happen after the change, can be overridden by later code, and makes the script’s behaviour depend on the environment.
+Best‑practice solutions are:
+1. **Avoid the name clash** – rename the local module (e.g., `my_spam.py`) so that it cannot be confused with the built‑in module.
+2. **Use an explicit loader** – if the name must stay the same, load the file directly with `importlib.machinery.SourceFileLoader` or `importlib.util.module_from_spec`, bypassing the normal import machinery.
+3. **Set the import path before the interpreter starts** – place `/opt/custom_lib` in the `PYTHONPATH` environment variable or use a virtual environment so that the desired directory is part of the initial `sys.path` and the script does not need to modify it.
+4. **Package the code** – place the local implementation inside a package (e.g., `my_pkg/spam.py`) and import it with an absolute import (`from my_pkg import spam`).
+These approaches respect the documented import order, eliminate reliance on runtime `sys.path` tweaks, and make the code portable and maintainable.</t>
+        </is>
+      </c>
+      <c r="M131" s="9" t="inlineStr">
+        <is>
+          <t>topic_4_modules.pdf_11, topic_4_modules.pdf_12</t>
+        </is>
+      </c>
+      <c r="N131" s="9" t="inlineStr">
+        <is>
+          <t>Import Search Order &amp; sys.path Best Practices</t>
+        </is>
+      </c>
+      <c r="O131" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P131" s="9" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="9" t="inlineStr">
+        <is>
+          <t>T4_017</t>
+        </is>
+      </c>
+      <c r="B132" s="9" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C132" s="9" t="inlineStr">
+        <is>
+          <t>Modules &amp; Packages</t>
+        </is>
+      </c>
+      <c r="D132" s="9" t="inlineStr">
+        <is>
+          <t>topic_4_modules.pdf</t>
+        </is>
+      </c>
+      <c r="E132" s="9" t="inlineStr">
+        <is>
+          <t>Evaluate</t>
+        </is>
+      </c>
+      <c r="F132" s="9" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G132" s="9" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="H132" s="9" t="inlineStr">
+        <is>
+          <t>Best Practice</t>
+        </is>
+      </c>
+      <c r="I132" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J132" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K132" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following Python code that imports the `fibo` module and uses its `fib` function in two different ways:
+```python
+import fibo
+# Approach A
+fibo.fib(100)
+# Approach B
+fib = fibo.fib
+fib(100)
+```
+Evaluate the two approaches with respect to readability, namespace management, and ease of maintenance in a larger code base. Which approach (or combination of approaches) represents best practice when you need to call a module function repeatedly, and why? Use only the information provided in the context.</t>
+        </is>
+      </c>
+      <c r="L132" s="9" t="inlineStr">
+        <is>
+          <t>Approach A (`fibo.fib(100)`) keeps the function call fully qualified, making it immediately clear that `fib` originates from the `fibo` module. This avoids accidental name clashes with any other `fib` defined elsewhere and preserves the module’s namespace, which is especially valuable in larger projects where many modules are imported.
+Approach B creates a local alias (`fib = fibo.fib`) and then calls `fib(100)`. The context explicitly notes that assigning a frequently‑used function to a local name is permissible and can reduce typing. This alias is appropriate when the function is called many times, because it shortens the code without losing the reference to the original implementation. However, the alias overwrites any existing name `fib` in the local scope, so developers must ensure it does not hide other identifiers.
+Best practice, therefore, is to use the fully‑qualified form (Approach A) for occasional calls and to create a local alias (Approach B) only when the function is used repeatedly throughout a module, as the context suggests. This balances readability and namespace safety with convenience.</t>
+        </is>
+      </c>
+      <c r="M132" s="9" t="inlineStr">
+        <is>
+          <t>topic_4_modules.pdf_2, topic_4_modules.pdf_3</t>
+        </is>
+      </c>
+      <c r="N132" s="9" t="inlineStr">
+        <is>
+          <t>Module import best practices</t>
+        </is>
+      </c>
+      <c r="O132" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P132" s="9" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="9" t="inlineStr">
+        <is>
+          <t>T4_018</t>
+        </is>
+      </c>
+      <c r="B133" s="9" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C133" s="9" t="inlineStr">
+        <is>
+          <t>Modules &amp; Packages</t>
+        </is>
+      </c>
+      <c r="D133" s="9" t="inlineStr">
+        <is>
+          <t>topic_4_modules.pdf</t>
+        </is>
+      </c>
+      <c r="E133" s="9" t="inlineStr">
+        <is>
+          <t>Evaluate</t>
+        </is>
+      </c>
+      <c r="F133" s="9" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G133" s="9" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="H133" s="9" t="inlineStr">
+        <is>
+          <t>Best Practice</t>
+        </is>
+      </c>
+      <c r="I133" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J133" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K133" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following Python script that uses the ``fibo`` module:
+```python
+# script.py
+import fibo
+from fibo import *
+from fibo import fib as fibonacci
+def compute():
+    # use fib from the wildcard import
+    fib(10)
+    # use fibonacci alias
+    fibonacci(15)
+    # use module‑qualified call
+    fibo.fib2(20)
+if __name__ == '__main__':
+    compute()
+```
+Evaluate the import strategy used in this script. Identify any practices that violate Python's recommended style for modules and packages. Propose a revised version of the imports that follows best‑practice guidelines, and explain why your revision improves code readability, maintainability, and avoids potential name conflicts.</t>
+        </is>
+      </c>
+      <c r="L133" s="9" t="inlineStr">
+        <is>
+          <t>The script mixes three different import styles and includes a ``from fibo import *`` statement, which is explicitly discouraged in the documentation because it pollutes the local namespace with an unknown set of names and can hide existing identifiers. Using both a wildcard import and an alias for the same function (``fib`` as ``fibonacci``) creates redundancy and makes it unclear which name should be used. A clearer, more maintainable approach is to import only the needed symbols explicitly or to import the module once and qualify all calls.
+A recommended revision is:
+```python
+# script.py
+import fibo
+# or, if only specific functions are needed:
+# from fibo import fib, fib2
+def compute():
+    fibo.fib(10)          # explicit module qualification
+    fibo.fib(15)          # reuse the same name; alias not required
+    fibo.fib2(20)
+if __name__ == '__main__':
+    compute()
+```
+This version eliminates the wildcard import, removes the unnecessary alias, and uses a single, consistent import style. The code is now easier to read because every function call is clearly associated with its source module, reducing the risk of name collisions and making future refactoring (e.g., swapping ``fibo`` for another implementation) straightforward.</t>
+        </is>
+      </c>
+      <c r="M133" s="9" t="inlineStr">
+        <is>
+          <t>topic_4_modules.pdf_6, topic_4_modules.pdf_7, topic_4_modules.pdf_8</t>
+        </is>
+      </c>
+      <c r="N133" s="9" t="inlineStr">
+        <is>
+          <t>Import Best Practices</t>
+        </is>
+      </c>
+      <c r="O133" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P133" s="9" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="9" t="inlineStr">
+        <is>
+          <t>T5_010</t>
+        </is>
+      </c>
+      <c r="B134" s="9" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
+      </c>
+      <c r="C134" s="9" t="inlineStr">
+        <is>
+          <t>File Input/Output</t>
+        </is>
+      </c>
+      <c r="D134" s="9" t="inlineStr">
+        <is>
+          <t>topic_5_input_output.pdf</t>
+        </is>
+      </c>
+      <c r="E134" s="9" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="F134" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G134" s="9" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="H134" s="9" t="inlineStr">
+        <is>
+          <t>Enumeration</t>
+        </is>
+      </c>
+      <c r="I134" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J134" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K134" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following Python snippet:
+```python
+import json
+data = [1, 'simple', 'list']
+json_str = json.dumps(data)
+with open('data.txt', 'w') as f:
+    json.dump(data, f)
+```
+Based on the code and the provided context, enumerate the two JSON module functions used for serializing data and briefly state what each function does.</t>
+        </is>
+      </c>
+      <c r="L134" s="9" t="inlineStr">
+        <is>
+          <t>1. **json.dumps()** – Serializes a Python object (e.g., a list) to a JSON‑formatted *string* and returns that string.
+2. **json.dump()** – Serializes a Python object to a JSON‑formatted representation *and writes it directly* to an open file object.</t>
+        </is>
+      </c>
+      <c r="M134" s="9" t="inlineStr">
+        <is>
+          <t>topic_5_input_output.pdf_29, topic_5_input_output.pdf_30, topic_5_input_output.pdf_31</t>
+        </is>
+      </c>
+      <c r="N134" s="9" t="inlineStr">
+        <is>
+          <t>JSON serialization functions</t>
+        </is>
+      </c>
+      <c r="O134" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P134" s="9" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="9" t="inlineStr">
+        <is>
+          <t>T5_011</t>
+        </is>
+      </c>
+      <c r="B135" s="9" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
+      </c>
+      <c r="C135" s="9" t="inlineStr">
+        <is>
+          <t>File Input/Output</t>
+        </is>
+      </c>
+      <c r="D135" s="9" t="inlineStr">
+        <is>
+          <t>topic_5_input_output.pdf</t>
+        </is>
+      </c>
+      <c r="E135" s="9" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="F135" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G135" s="9" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="H135" s="9" t="inlineStr">
+        <is>
+          <t>Enumeration</t>
+        </is>
+      </c>
+      <c r="I135" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J135" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K135" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following Python code that writes formatted strings to a file:
+```python
+data = {'name': 'Alice', 'score': 93.4567}
+with open('results.txt', 'w') as f:
+    f.write(f"{data['name']:&lt;10} ==&gt; {data['score']:.2f}\n")
+    f.write(f"{data['name']!r} has score {data['score']!s}\n")
+```
+Enumerate all distinct formatting options (field‑width specifier, precision specifier, conversion flags, and the = specifier) that appear in the f‑strings used in this snippet, as described in the provided context.</t>
+        </is>
+      </c>
+      <c r="L135" s="9" t="inlineStr">
+        <is>
+          <t>The f‑strings in the snippet use four distinct formatting options described in the context:
+1. A field‑width specifier `:&lt;10` that makes the name field at least 10 characters wide.
+2. A precision specifier `:.2f` that rounds the score to two decimal places.
+3. The conversion flag `!r` which applies `repr()` to the name value.
+4. The conversion flag `!s` which applies `str()` to the score value.
+(The `=` specifier is mentioned in the context but does not appear in this code.)</t>
+        </is>
+      </c>
+      <c r="M135" s="9" t="inlineStr">
+        <is>
+          <t>topic_5_input_output.pdf_7, topic_5_input_output.pdf_8, topic_5_input_output.pdf_9, topic_5_input_output.pdf_10</t>
+        </is>
+      </c>
+      <c r="N135" s="9" t="inlineStr">
+        <is>
+          <t>f-string formatting options</t>
+        </is>
+      </c>
+      <c r="O135" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P135" s="9" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="9" t="inlineStr">
+        <is>
+          <t>T5_012</t>
+        </is>
+      </c>
+      <c r="B136" s="9" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
+      </c>
+      <c r="C136" s="9" t="inlineStr">
+        <is>
+          <t>File Input/Output</t>
+        </is>
+      </c>
+      <c r="D136" s="9" t="inlineStr">
+        <is>
+          <t>topic_5_input_output.pdf</t>
+        </is>
+      </c>
+      <c r="E136" s="9" t="inlineStr">
+        <is>
+          <t>Evaluate</t>
+        </is>
+      </c>
+      <c r="F136" s="9" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G136" s="9" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H136" s="9" t="inlineStr">
+        <is>
+          <t>Best Practice</t>
+        </is>
+      </c>
+      <c r="I136" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J136" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K136" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Consider two snippets that write the contents of a dictionary to a text file. Both produce the same output, but they use different formatting techniques.
+Snippet A:
+```python
+table = {'Sjoerd': 4127, 'Jack': 4098, 'Dcab': 8637678}
+with open('scores.txt', 'w') as f:
+    f.write('Jack: {0[Jack]:d}; Sjoerd: {0[Sjoerd]:d}; Dcab: {0[Dcab]:d}\n'.format(table))
+```
+Snippet B:
+```python
+table = {'Sjoerd': 4127, 'Jack': 4098, 'Dcab': 8637678}
+with open('scores.txt', 'w') as f:
+    f.write('Jack: {Jack:d}; Sjoerd: {Sjoerd:d}; Dcab: {Dcab:d}\n'.format(**table))
+```
+Evaluate which snippet represents best practice for file input/output in Python. In your evaluation discuss readability, maintainability, and potential error‑prone aspects of each approach, and state which one you would recommend for production code.
+</t>
+        </is>
+      </c>
+      <c r="L136" s="9" t="inlineStr">
+        <is>
+          <t>Snippet B, which uses the ** unpacking operator, is the better practice. It keeps the format string clean and readable because the placeholders match the dictionary keys directly, eliminating the repetitive ``{0[key]}`` syntax seen in Snippet A. This reduces visual clutter and makes it easier to spot missing or misspelled keys. Moreover, when the dictionary’s contents change (e.g., adding or removing entries), the format string in Snippet B needs only the placeholders that are actually required, whereas Snippet A tightly couples the string to the positional ``0`` reference, increasing the chance of a ``KeyError`` if a key is absent. Both snippets will raise a ``KeyError`` for missing keys, but the ** form makes the relationship between data and format explicit, aiding future maintenance and code reviews. Therefore, for production‑level file I/O, Snippet B is recommended for its superior readability and maintainability.</t>
+        </is>
+      </c>
+      <c r="M136" s="9" t="inlineStr">
+        <is>
+          <t>topic_5_input_output.pdf_12</t>
+        </is>
+      </c>
+      <c r="N136" s="9" t="inlineStr">
+        <is>
+          <t>String Formatting Best Practices</t>
+        </is>
+      </c>
+      <c r="O136" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P136" s="9" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="9" t="inlineStr">
+        <is>
+          <t>T5_013</t>
+        </is>
+      </c>
+      <c r="B137" s="9" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
+      </c>
+      <c r="C137" s="9" t="inlineStr">
+        <is>
+          <t>File Input/Output</t>
+        </is>
+      </c>
+      <c r="D137" s="9" t="inlineStr">
+        <is>
+          <t>topic_5_input_output.pdf</t>
+        </is>
+      </c>
+      <c r="E137" s="9" t="inlineStr">
+        <is>
+          <t>Evaluate</t>
+        </is>
+      </c>
+      <c r="F137" s="9" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G137" s="9" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="H137" s="9" t="inlineStr">
+        <is>
+          <t>Best Practice</t>
+        </is>
+      </c>
+      <c r="I137" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J137" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K137" s="9" t="inlineStr">
+        <is>
+          <t>You are tasked with persisting a list of user settings that may need to be read by a web service written in JavaScript. Two developers propose the following snippets:
+```python
+# Developer A – JSON (correct usage)
+import json
+settings = [{"theme": "dark", "notifications": True}, {"theme": "light", "notifications": False}]
+with open('settings.json', 'w', encoding='utf-8') as f:
+    json.dump(settings, f)
+```
+```python
+# Developer B – Pickle (problematic usage)
+import pickle
+settings = [{"theme": "dark", "notifications": True}, {"theme": "light", "notifications": False}]
+with open('settings.pkl', 'w') as f:  # note text mode
+    pickle.dump(settings, f)
+```
+Evaluate the two approaches and recommend the best‑practice method for saving these settings. In your answer, consider cross‑language compatibility, security implications, and proper file handling (mode and encoding).</t>
+        </is>
+      </c>
+      <c r="L137" s="9" t="inlineStr">
+        <is>
+          <t>Using JSON (Developer A) is the best practice for this scenario. JSON produces a UTF‑8 encoded text file that can be read by any language, including JavaScript, and it does not execute code when deserialized, so it avoids the security risk inherent to pickle. The code correctly opens the file in text mode with explicit UTF‑8 encoding, which satisfies the requirement that JSON files be UTF‑8. 
+Pickle (Developer B) is unsuitable here: it serializes Python‑specific objects, making the file unreadable by non‑Python programs, and unpickling untrusted data can execute arbitrary code, posing a serious security vulnerability. Moreover, the file is opened in text mode; pickle data should be written in binary mode ('wb') to avoid data corruption. Therefore, the recommended approach is to use the JSON snippet as shown, ensuring the file is opened with `encoding='utf-8'` and using `json.dump` for serialization.</t>
+        </is>
+      </c>
+      <c r="M137" s="9" t="inlineStr">
+        <is>
+          <t>topic_5_input_output.pdf_32, topic_5_input_output.pdf_33</t>
+        </is>
+      </c>
+      <c r="N137" s="9" t="inlineStr">
+        <is>
+          <t>Secure serialization best practice</t>
+        </is>
+      </c>
+      <c r="O137" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P137" s="9" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="9" t="inlineStr">
+        <is>
+          <t>T5_014</t>
+        </is>
+      </c>
+      <c r="B138" s="9" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
+      </c>
+      <c r="C138" s="9" t="inlineStr">
+        <is>
+          <t>File Input/Output</t>
+        </is>
+      </c>
+      <c r="D138" s="9" t="inlineStr">
+        <is>
+          <t>topic_5_input_output.pdf</t>
+        </is>
+      </c>
+      <c r="E138" s="9" t="inlineStr">
+        <is>
+          <t>Evaluate</t>
+        </is>
+      </c>
+      <c r="F138" s="9" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G138" s="9" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="H138" s="9" t="inlineStr">
+        <is>
+          <t>Best Practice</t>
+        </is>
+      </c>
+      <c r="I138" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J138" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K138" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Consider the following two Python code snippets that read all lines from a source text file, convert each line to uppercase, and write the results to a destination file.
+Snippet A (does not use best‑practice constructs):
+```python
+src = open('input.txt')
+lines = src.readlines()
+src.close()
+dst = open('output.txt', 'w')
+for line in lines:
+    dst.write(line.upper())
+# forgetting to close the destination file
+```
+Snippet B (uses recommended practices):
+```python
+with open('input.txt', encoding='utf-8') as src:
+    lines = src.readlines()
+with open('output.txt', mode='w', encoding='utf-8') as dst:
+    for line in lines:
+        dst.write(line.upper())
+```
+**Question:** Evaluate which snippet follows the best practices for file input/output in Python. Identify the specific shortcomings of the other snippet and explain how they could affect program correctness, resource management, or portability.
+</t>
+        </is>
+      </c>
+      <c r="L138" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Snippet B follows the best‑practice guidelines. It uses the `with` statement for both files, guaranteeing that each file is automatically closed even if an exception occurs, which prevents resource leaks. It also explicitly specifies `encoding='utf-8'`, avoiding reliance on the platform‑dependent default encoding and ensuring correct handling of non‑ASCII characters. The mode is given as `'w'` (text mode) appropriate for writing strings.
+Snippet A has several problems: it opens files without `with`, so the source file is manually closed but the destination file is never closed, risking file‑descriptor leaks. It omits an explicit `encoding`, so the default platform encoding is used; on systems where the default is not UTF‑8, reading or writing Unicode data may raise errors or corrupt text. Additionally, forgetting to close `dst` means buffered data may not be flushed to disk, leading to incomplete output. These issues affect portability, correctness with Unicode data, and reliable resource cleanup.
+</t>
+        </is>
+      </c>
+      <c r="M138" s="9" t="inlineStr">
+        <is>
+          <t>topic_5_input_output.pdf_19, topic_5_input_output.pdf_20, topic_5_input_output.pdf_21</t>
+        </is>
+      </c>
+      <c r="N138" s="9" t="inlineStr">
+        <is>
+          <t>File handling best practices</t>
+        </is>
+      </c>
+      <c r="O138" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P138" s="9" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="9" t="inlineStr">
+        <is>
+          <t>T5_015</t>
+        </is>
+      </c>
+      <c r="B139" s="9" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
+      </c>
+      <c r="C139" s="9" t="inlineStr">
+        <is>
+          <t>File Input/Output</t>
+        </is>
+      </c>
+      <c r="D139" s="9" t="inlineStr">
+        <is>
+          <t>topic_5_input_output.pdf</t>
+        </is>
+      </c>
+      <c r="E139" s="9" t="inlineStr">
+        <is>
+          <t>Evaluate</t>
+        </is>
+      </c>
+      <c r="F139" s="9" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G139" s="9" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="H139" s="9" t="inlineStr">
+        <is>
+          <t>Best Practice</t>
+        </is>
+      </c>
+      <c r="I139" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J139" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K139" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following two Python snippets that attempt to write a dictionary to a JSON file.
+Snippet A:
+```python
+import json
+data = {"name": "Alice", "age": 30, "scores": [85, 92, 78]}
+f = open('data.json', 'w')
+json_string = json.dumps(data)
+f.write(json_string)
+f.close()
+```
+Snippet B:
+```python
+import json
+data = {"name": "Alice", "age": 30, "scores": [85, 92, 78]}
+with open('data.json', 'w', encoding='utf-8') as f:
+    json.dump(data, f)
+```
+Evaluate which snippet follows best practices for file I/O and JSON serialization in Python. Identify any problems in the non‑optimal snippet, explain why they matter, and provide a corrected version of that snippet that adheres to best practices.</t>
+        </is>
+      </c>
+      <c r="L139" s="9" t="inlineStr">
+        <is>
+          <t>Snippet B follows best practices. It uses a with‑statement, guaranteeing the file is closed even if an exception occurs, and explicitly sets encoding='utf-8', which is required for JSON files. It also calls json.dump directly, avoiding an unnecessary intermediate string and reducing memory overhead.
+Snippet A has three issues: (1) it opens the file without specifying UTF‑8, which can corrupt non‑ASCII characters; (2) it manually converts the object with json.dumps and writes the string, adding an extra step and potential encoding mismatches; (3) it relies on an explicit f.close(), which will not run if an error occurs before the call, risking a resource leak.
+A corrected version of Snippet A that meets best‑practice standards is:
+```python
+import json
+data = {"name": "Alice", "age": 30, "scores": [85, 92, 78]}
+with open('data.json', 'w', encoding='utf-8') as f:
+    json.dump(data, f)
+```</t>
+        </is>
+      </c>
+      <c r="M139" s="9" t="inlineStr">
+        <is>
+          <t>topic_5_input_output.pdf_30, topic_5_input_output.pdf_31, topic_5_input_output.pdf_32</t>
+        </is>
+      </c>
+      <c r="N139" s="9" t="inlineStr">
+        <is>
+          <t>JSON file handling best practices</t>
+        </is>
+      </c>
+      <c r="O139" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P139" s="9" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="9" t="inlineStr">
+        <is>
+          <t>T6_018</t>
+        </is>
+      </c>
+      <c r="B140" s="9" t="inlineStr">
+        <is>
+          <t>T6</t>
+        </is>
+      </c>
+      <c r="C140" s="9" t="inlineStr">
+        <is>
+          <t>Errors &amp; Exceptions</t>
+        </is>
+      </c>
+      <c r="D140" s="9" t="inlineStr">
+        <is>
+          <t>topic_7_errors_exceptions.pdf</t>
+        </is>
+      </c>
+      <c r="E140" s="9" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="F140" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G140" s="9" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="H140" s="9" t="inlineStr">
+        <is>
+          <t>Enumeration</t>
+        </is>
+      </c>
+      <c r="I140" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J140" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K140" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following Python code that collects exceptions into an ExceptionGroup and adds a note to each caught exception:
+```python
+def f():
+    raise OSError('operation failed')
+excs = []
+for i in range(3):
+    try:
+        f()
+    except Exception as e:
+        e.add_note(f'Happened in Iteration {i+1}')
+        excs.append(e)
+raise ExceptionGroup('We have some problems', excs)
+```
+List, in order, the note strings that will be attached to each sub‑exception in the resulting ExceptionGroup.</t>
+        </is>
+      </c>
+      <c r="L140" s="9" t="inlineStr">
+        <is>
+          <t>The notes attached to the three sub‑exceptions are:
+1. "Happened in Iteration 1"
+2. "Happened in Iteration 2"
+3. "Happened in Iteration 3"</t>
+        </is>
+      </c>
+      <c r="M140" s="9" t="inlineStr">
+        <is>
+          <t>topic_7_errors_exceptions.pdf_35, topic_7_errors_exceptions.pdf_36, topic_7_errors_exceptions.pdf_37</t>
+        </is>
+      </c>
+      <c r="N140" s="9" t="inlineStr">
+        <is>
+          <t>Exception notes in ExceptionGroup</t>
+        </is>
+      </c>
+      <c r="O140" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P140" s="9" t="n"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="9" t="inlineStr">
+        <is>
+          <t>T6_019</t>
+        </is>
+      </c>
+      <c r="B141" s="9" t="inlineStr">
+        <is>
+          <t>T6</t>
+        </is>
+      </c>
+      <c r="C141" s="9" t="inlineStr">
+        <is>
+          <t>Errors &amp; Exceptions</t>
+        </is>
+      </c>
+      <c r="D141" s="9" t="inlineStr">
+        <is>
+          <t>topic_7_errors_exceptions.pdf</t>
+        </is>
+      </c>
+      <c r="E141" s="9" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="F141" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G141" s="9" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="H141" s="9" t="inlineStr">
+        <is>
+          <t>Enumeration</t>
+        </is>
+      </c>
+      <c r="I141" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J141" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K141" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following two code snippets:
+```python
+# Snippet A
+def func():
+    raise ConnectionError
+try:
+    func()
+except ConnectionError as exc:
+    raise RuntimeError('Failed to open database') from exc
+```
+```python
+# Snippet B
+try:
+    open('database.sqlite')
+except OSError:
+    raise RuntimeError from None
+```
+Based on the context, enumerate:
+1. The effect of the `from exc` clause in Snippet A on the traceback.
+2. The effect of the `from None` clause in Snippet B on the traceback.
+List each effect as a separate bullet point.</t>
+        </is>
+      </c>
+      <c r="L141" s="9" t="inlineStr">
+        <is>
+          <t>- In Snippet A, `from exc` creates explicit exception chaining, so the traceback shows both the original `ConnectionError` and the new `RuntimeError`, with a line stating “The above exception was the direct cause of the following exception.”
+- In Snippet B, `from None` disables automatic exception chaining, so the traceback displays only the `RuntimeError` without any reference to the original `OSError`.</t>
+        </is>
+      </c>
+      <c r="M141" s="9" t="inlineStr">
+        <is>
+          <t>topic_7_errors_exceptions.pdf_19, topic_7_errors_exceptions.pdf_20, topic_7_errors_exceptions.pdf_21, topic_7_errors_exceptions.pdf_22</t>
+        </is>
+      </c>
+      <c r="N141" s="9" t="inlineStr">
+        <is>
+          <t>Exception chaining</t>
+        </is>
+      </c>
+      <c r="O141" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P141" s="9" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="9" t="inlineStr">
+        <is>
+          <t>T6_020</t>
+        </is>
+      </c>
+      <c r="B142" s="9" t="inlineStr">
+        <is>
+          <t>T6</t>
+        </is>
+      </c>
+      <c r="C142" s="9" t="inlineStr">
+        <is>
+          <t>Errors &amp; Exceptions</t>
+        </is>
+      </c>
+      <c r="D142" s="9" t="inlineStr">
+        <is>
+          <t>topic_7_errors_exceptions.pdf</t>
+        </is>
+      </c>
+      <c r="E142" s="9" t="inlineStr">
+        <is>
+          <t>Evaluate</t>
+        </is>
+      </c>
+      <c r="F142" s="9" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G142" s="9" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H142" s="9" t="inlineStr">
+        <is>
+          <t>Best Practice</t>
+        </is>
+      </c>
+      <c r="I142" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J142" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K142" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following Python code:
+```python
+while True print('Hello world')
+```
+When this code is executed, Python raises a SyntaxError and displays the line with a caret (^) under the word `print`. According to the description in the context, evaluate which of the following debugging approaches follows best practice and justify your choice:
+1. Assume the error is at the `print` token because the caret points there, and add a colon after `print`.
+2. Recognize that the caret indicates where the parser detected the problem, and check the code immediately before `print` for a missing colon.
+Provide your evaluation and reasoning.</t>
+        </is>
+      </c>
+      <c r="L142" s="9" t="inlineStr">
+        <is>
+          <t>The second approach follows best practice. The context explains that the parser’s caret points to the location where it *detected* the syntax error, which is not necessarily the exact spot that needs fixing. In the example, the missing colon before `print` causes the parser to flag `print`, so the correct fix is to add the colon after `while True`. Therefore, examining the code preceding the highlighted token (the missing colon) is the proper way to locate and correct the error.</t>
+        </is>
+      </c>
+      <c r="M142" s="9" t="inlineStr">
+        <is>
+          <t>topic_7_errors_exceptions.pdf_1</t>
+        </is>
+      </c>
+      <c r="N142" s="9" t="inlineStr">
+        <is>
+          <t>Interpreting SyntaxError messages</t>
+        </is>
+      </c>
+      <c r="O142" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P142" s="9" t="n"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="9" t="inlineStr">
+        <is>
+          <t>T6_021</t>
+        </is>
+      </c>
+      <c r="B143" s="9" t="inlineStr">
+        <is>
+          <t>T6</t>
+        </is>
+      </c>
+      <c r="C143" s="9" t="inlineStr">
+        <is>
+          <t>Errors &amp; Exceptions</t>
+        </is>
+      </c>
+      <c r="D143" s="9" t="inlineStr">
+        <is>
+          <t>topic_7_errors_exceptions.pdf</t>
+        </is>
+      </c>
+      <c r="E143" s="9" t="inlineStr">
+        <is>
+          <t>Evaluate</t>
+        </is>
+      </c>
+      <c r="F143" s="9" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G143" s="9" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="H143" s="9" t="inlineStr">
+        <is>
+          <t>Best Practice</t>
+        </is>
+      </c>
+      <c r="I143" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J143" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K143" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following Python function that processes user input and performs division:
+```python
+def compute():
+    try:
+        x = input("Enter numerator: ")
+        y = input("Enter denominator: ")
+        result = int(x) / int(y)
+        print("Result:", result)
+    except:
+        print("An error occurred.")
+    finally:
+        print("Computation finished.")
+```
+Evaluate the error‑handling approach used in this code. Using the context about exception types (e.g., `NameError`, `TypeError`, `ZeroDivisionError`) and how they are reported, identify **at least three** shortcomings of the current `except` block. Then rewrite the function so that it follows best‑practice guidelines for handling these specific exceptions (and optionally `ValueError` for bad casts). Explain why your revised version is a better practice for debugging and user feedback.</t>
+        </is>
+      </c>
+      <c r="L143" s="9" t="inlineStr">
+        <is>
+          <t>**Shortcomings of the original `except` block**
+1. **Bare except hides the exception type** – the traceback’s last line (e.g., `NameError`, `TypeError`) is never shown, so the programmer cannot know whether the problem was an undefined name, a bad concatenation, or a division by zero. This contradicts the context that the exception type is printed as part of the error message and is useful for diagnosing the error.
+2. **All errors are treated the same** – the message "An error occurred" gives no guidance to the user about what went wrong (e.g., non‑numeric input vs. division by zero). Best‑practice recommends handling each expected exception separately so that feedback can be specific.
+3. **Potentially catches unrelated system errors** – a bare `except:` also traps `KeyboardInterrupt`, `SystemExit`, and other critical exceptions, making the program harder to stop or debug.
+**Revised function following best practices**
+```python
+def compute():
+    try:
+        x = input("Enter numerator: ")
+        y = input("Enter denominator: ")
+        result = int(x) / int(y)
+        print("Result:", result)
+    except ZeroDivisionError:
+        print("Error: cannot divide by zero.")
+    except ValueError:
+        # raised when int() cannot convert a non‑numeric string
+        print("Error: please enter valid integers.")
+    except TypeError:
+        # would occur if, for example, a string were added to an int
+        print("Error: type mismatch in the operation.")
+    except NameError:
+        # unlikely here but shown for completeness per the context
+        print("Error: a variable was used before being defined.")
+    finally:
+        print("Computation finished.")
+```
+**Why this is preferable**
+- **Specificity**: Each `except` clause matches a concrete exception type, allowing the program to report the exact problem, which aligns with the context’s emphasis on the exception type being part of the error message.
+- **Safety**: By not using a bare `except`, critical system exceptions propagate normally, preserving expected interpreter behavior.
+- **Maintainability**: Future readers can see at a glance which error conditions are anticipated, making debugging easier and encouraging the practice of catching only those exceptions that the code can meaningfully handle.
+- **User experience**: Tailored messages guide the user to correct the input rather than presenting a vague "An error occurred" message.</t>
+        </is>
+      </c>
+      <c r="M143" s="9" t="inlineStr">
+        <is>
+          <t>topic_7_errors_exceptions.pdf_3, topic_7_errors_exceptions.pdf_4</t>
+        </is>
+      </c>
+      <c r="N143" s="9" t="inlineStr">
+        <is>
+          <t>Exception handling best practices</t>
+        </is>
+      </c>
+      <c r="O143" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P143" s="9" t="n"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="9" t="inlineStr">
+        <is>
+          <t>T6_022</t>
+        </is>
+      </c>
+      <c r="B144" s="9" t="inlineStr">
+        <is>
+          <t>T6</t>
+        </is>
+      </c>
+      <c r="C144" s="9" t="inlineStr">
+        <is>
+          <t>Errors &amp; Exceptions</t>
+        </is>
+      </c>
+      <c r="D144" s="9" t="inlineStr">
+        <is>
+          <t>topic_7_errors_exceptions.pdf</t>
+        </is>
+      </c>
+      <c r="E144" s="9" t="inlineStr">
+        <is>
+          <t>Evaluate</t>
+        </is>
+      </c>
+      <c r="F144" s="9" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G144" s="9" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="H144" s="9" t="inlineStr">
+        <is>
+          <t>Best Practice</t>
+        </is>
+      </c>
+      <c r="I144" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J144" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K144" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following two functions that attempt to open a database file and translate any OSError into a RuntimeError.
+```python
+def open_db_keep():
+    try:
+        open('database.sqlite')
+    except OSError as exc:
+        raise RuntimeError('Failed to open database') from exc
+def open_db_suppress():
+    try:
+        open('database.sqlite')
+    except OSError:
+        raise RuntimeError('Failed to open database') from None
+```
+You are reviewing code for a large project. Evaluate which of the two implementations follows best practice for exception handling in this context, and justify your recommendation with reference to exception chaining semantics, debugging usefulness, and API design considerations.</t>
+        </is>
+      </c>
+      <c r="L144" s="9" t="inlineStr">
+        <is>
+          <t>The implementation that uses ``raise RuntimeError('Failed to open database') from exc`` (``open_db_keep``) follows best practice in most production code. By chaining the new ``RuntimeError`` to the original ``OSError`` the traceback retains the low‑level cause, which is invaluable for debugging and for any higher‑level error‑handling logic that may want to inspect the original exception type or message. This aligns with the Python documentation’s recommendation to preserve the direct cause unless there is a compelling reason to hide it.
+Using ``from None`` (as in ``open_db_suppress``) deliberately suppresses the chaining. It should be reserved for situations where exposing the underlying exception would leak implementation details, create security concerns, or add noise to the public API. In the simple case of opening a database file, callers typically benefit from seeing that the failure originated from an ``OSError`` (e.g., file not found or permission denied). Therefore, ``open_db_keep`` is the preferred approach.
+If a custom exception were defined, it should inherit from ``Exception`` and follow the “*Error*” naming convention (e.g., ``DatabaseOpenError``), but the chaining decision remains the same: preserve the original exception with ``from exc`` unless intentional suppression is required.</t>
+        </is>
+      </c>
+      <c r="M144" s="9" t="inlineStr">
+        <is>
+          <t>topic_7_errors_exceptions.pdf_19, topic_7_errors_exceptions.pdf_20, topic_7_errors_exceptions.pdf_21</t>
+        </is>
+      </c>
+      <c r="N144" s="9" t="inlineStr">
+        <is>
+          <t>Exception Chaining Best Practices</t>
+        </is>
+      </c>
+      <c r="O144" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P144" s="9" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="9" t="inlineStr">
+        <is>
+          <t>T6_023</t>
+        </is>
+      </c>
+      <c r="B145" s="9" t="inlineStr">
+        <is>
+          <t>T6</t>
+        </is>
+      </c>
+      <c r="C145" s="9" t="inlineStr">
+        <is>
+          <t>Errors &amp; Exceptions</t>
+        </is>
+      </c>
+      <c r="D145" s="9" t="inlineStr">
+        <is>
+          <t>topic_7_errors_exceptions.pdf</t>
+        </is>
+      </c>
+      <c r="E145" s="9" t="inlineStr">
+        <is>
+          <t>Evaluate</t>
+        </is>
+      </c>
+      <c r="F145" s="9" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G145" s="9" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="H145" s="9" t="inlineStr">
+        <is>
+          <t>Best Practice</t>
+        </is>
+      </c>
+      <c r="I145" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J145" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K145" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following Python snippet that repeatedly prompts the user for a number:
+```python
+while True:
+    try:
+        x = int(input("Please enter a number: "))
+        break
+    except ValueError:
+        print("Oops! That was no valid number. Try again...")
+```
+Evaluate this code from a best‑practice standpoint. Identify any shortcomings in its exception handling or user‑input strategy, and propose concrete improvements (e.g., handling additional exceptions, limiting attempts, separating concerns, using an else clause). Justify why your suggested changes represent better practice.</t>
+        </is>
+      </c>
+      <c r="L145" s="9" t="inlineStr">
+        <is>
+          <t>The snippet correctly catches a ValueError when the user enters non‑numeric text, but it has several best‑practice issues. First, it ignores other possible exceptions from `input`, such as `EOFError` or `KeyboardInterrupt`, which would terminate the program abruptly; handling them (e.g., by cleanly exiting or prompting again) makes the program more robust. Second, the infinite `while True` loop relies on a `break` inside the `try` block; placing the successful conversion in an `else` clause clarifies the control flow:
+```python
+while True:
+    try:
+        x = int(input("Please enter a number: "))
+    except ValueError:
+        print("Oops! That was no valid number. Try again...")
+    except (EOFError, KeyboardInterrupt):
+        print("Input cancelled; exiting.")
+        sys.exit()
+    else:
+        break
+```
+Third, an unbounded loop can trap a user who repeatedly fails; adding a maximum‑attempt counter (e.g., 5 tries) and raising a custom exception after the limit improves usability. Finally, encapsulating the logic in a function (`def read_int(prompt): …`) separates concerns and makes the code reusable and testable. These changes enhance readability, safety, and maintainability, aligning the code with Python’s recommended exception‑handling practices.</t>
+        </is>
+      </c>
+      <c r="M145" s="9" t="inlineStr">
+        <is>
+          <t>topic_7_errors_exceptions.pdf_6, topic_7_errors_exceptions.pdf_7, topic_7_errors_exceptions.pdf_8</t>
+        </is>
+      </c>
+      <c r="N145" s="9" t="inlineStr">
+        <is>
+          <t>Exception handling best practices</t>
+        </is>
+      </c>
+      <c r="O145" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P145" s="9" t="n"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="9" t="inlineStr">
+        <is>
+          <t>T7_022</t>
+        </is>
+      </c>
+      <c r="B146" s="9" t="inlineStr">
         <is>
           <t>T7</t>
         </is>
       </c>
-      <c r="C107" s="7" t="inlineStr">
+      <c r="C146" s="9" t="inlineStr">
         <is>
           <t>Object-Oriented Programming</t>
         </is>
       </c>
-      <c r="D107" s="7" t="inlineStr">
+      <c r="D146" s="9" t="inlineStr">
         <is>
           <t>topic_7_oop.pdf</t>
         </is>
       </c>
-      <c r="E107" s="7" t="inlineStr">
+      <c r="E146" s="9" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="F146" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G146" s="9" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="H146" s="9" t="inlineStr">
+        <is>
+          <t>Enumeration</t>
+        </is>
+      </c>
+      <c r="I146" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J146" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K146" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following Python code snippet:
+```python
+import math as modname
+# assign a new attribute
+modname.the_answer = 42
+# delete the attribute
+del modname.the_answer
+```
+Based on the supplied context, enumerate all statements that are true about:
+1. module attributes;
+2. the effect of the assignment and deletion shown; and
+3. the lifetimes of the built‑in, global, and local namespaces.</t>
+        </is>
+      </c>
+      <c r="L146" s="9" t="inlineStr">
+        <is>
+          <t>1. Module attributes are writable – you can assign to them (e.g., `modname.the_answer = 42`).
+2. Module attributes can be deleted with `del` (e.g., `del modname.the_answer`).
+3. The built‑in namespace is created when the interpreter starts and never deleted.
+4. A module’s global namespace is created when the module definition is read and normally lasts until the interpreter quits.
+5. The `__main__` module has its own global namespace, created in the same way as any other module.
+6. A function’s local namespace is created each time the function is called and is deleted when the function returns (or an unhandled exception propagates).</t>
+        </is>
+      </c>
+      <c r="M146" s="9" t="inlineStr">
+        <is>
+          <t>topic_7_oop.pdf_8, topic_7_oop.pdf_9, topic_7_oop.pdf_10</t>
+        </is>
+      </c>
+      <c r="N146" s="9" t="inlineStr">
+        <is>
+          <t>Module attributes and namespace lifetimes</t>
+        </is>
+      </c>
+      <c r="O146" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P146" s="9" t="n"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="9" t="inlineStr">
+        <is>
+          <t>T7_023</t>
+        </is>
+      </c>
+      <c r="B147" s="9" t="inlineStr">
+        <is>
+          <t>T7</t>
+        </is>
+      </c>
+      <c r="C147" s="9" t="inlineStr">
+        <is>
+          <t>Object-Oriented Programming</t>
+        </is>
+      </c>
+      <c r="D147" s="9" t="inlineStr">
+        <is>
+          <t>topic_7_oop.pdf</t>
+        </is>
+      </c>
+      <c r="E147" s="9" t="inlineStr">
+        <is>
+          <t>Understand</t>
+        </is>
+      </c>
+      <c r="F147" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G147" s="9" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="H147" s="9" t="inlineStr">
+        <is>
+          <t>Enumeration</t>
+        </is>
+      </c>
+      <c r="I147" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J147" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K147" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following Python class definition:
+```python
+class Bag:
+    def __init__(self):
+        self.data = []
+    def add(self, x):
+        self.data.append(x)
+    def addtwice(self, x):
+        self.add(x)
+        self.add(x)
+```
+Based solely on the provided context, enumerate each method defined in the Bag class and briefly state the purpose of each method.</t>
+        </is>
+      </c>
+      <c r="L147" s="9" t="inlineStr">
+        <is>
+          <t>- __init__: the constructor that creates a new Bag instance and initializes an empty list stored in the attribute `data`.
+- add: appends a given element `x` to the bag's internal list `data`.
+- addtwice: calls `add` twice, thereby inserting the same element `x` into `data` two times.</t>
+        </is>
+      </c>
+      <c r="M147" s="9" t="inlineStr">
+        <is>
+          <t>topic_7_oop.pdf_37, topic_7_oop.pdf_38, topic_7_oop.pdf_39, topic_7_oop.pdf_40</t>
+        </is>
+      </c>
+      <c r="N147" s="9" t="inlineStr">
+        <is>
+          <t>Bag class method enumeration</t>
+        </is>
+      </c>
+      <c r="O147" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="P147" s="9" t="n"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="9" t="inlineStr">
+        <is>
+          <t>T7_024</t>
+        </is>
+      </c>
+      <c r="B148" s="9" t="inlineStr">
+        <is>
+          <t>T7</t>
+        </is>
+      </c>
+      <c r="C148" s="9" t="inlineStr">
+        <is>
+          <t>Object-Oriented Programming</t>
+        </is>
+      </c>
+      <c r="D148" s="9" t="inlineStr">
+        <is>
+          <t>topic_7_oop.pdf</t>
+        </is>
+      </c>
+      <c r="E148" s="9" t="inlineStr">
         <is>
           <t>Evaluate</t>
         </is>
       </c>
-      <c r="F107" s="7" t="inlineStr">
+      <c r="F148" s="9" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
       </c>
-      <c r="G107" s="7" t="inlineStr">
-        <is>
-          <t>R4</t>
-        </is>
-      </c>
-      <c r="H107" s="7" t="inlineStr">
+      <c r="G148" s="9" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="H148" s="9" t="inlineStr">
         <is>
           <t>Best Practice</t>
         </is>
       </c>
-      <c r="I107" s="7" t="inlineStr">
+      <c r="I148" s="9" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
       </c>
-      <c r="J107" s="7" t="inlineStr">
+      <c r="J148" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K148" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following two Python implementations that demonstrate method overriding in a derived class. Both aim to extend the behavior of `Base.process()`.
+```python
+class Base:
+    def process(self, data):
+        print('Base processing', data)
+        return data * 2
+# Implementation A
+class DerivedA(Base):
+    def process(self, data):
+        # Extend base behavior
+        result = Base.process(self, data)  # direct call to the base class
+        print('DerivedA additional step')
+        return result + 1
+# Implementation B
+class DerivedB(Base):
+    def process(self, data):
+        # Extend base behavior
+        result = super().process(data)   # use super()
+        print('DerivedB additional step')
+        return result + 1
+```
+Which implementation follows best practice for overriding methods in Python, and why? If either implementation has a flaw, show the corrected code line(s).</t>
+        </is>
+      </c>
+      <c r="L148" s="9" t="inlineStr">
+        <is>
+          <t>Implementation B follows best practice because it uses `super().process(data)` to invoke the base‑class method. Using `super()` respects the method resolution order, works correctly with multiple inheritance, and avoids hard‑coding the parent class name. Implementation A calls `Base.process(self, data)` directly, which bypasses the MRO and can break in more complex inheritance hierarchies. The corrected line for Implementation A would be:
+```python
+result = super().process(data)
+```</t>
+        </is>
+      </c>
+      <c r="M148" s="9" t="inlineStr">
+        <is>
+          <t>topic_7_oop.pdf_40</t>
+        </is>
+      </c>
+      <c r="N148" s="9" t="inlineStr">
+        <is>
+          <t>Method Overriding Best Practices</t>
+        </is>
+      </c>
+      <c r="O148" s="9" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="K107" s="4" t="n"/>
-      <c r="L107" s="4" t="n"/>
-      <c r="M107" s="4" t="n"/>
-      <c r="N107" s="4" t="n"/>
-      <c r="O107" s="7" t="inlineStr">
+      <c r="P148" s="9" t="n"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="9" t="inlineStr">
+        <is>
+          <t>T7_025</t>
+        </is>
+      </c>
+      <c r="B149" s="9" t="inlineStr">
+        <is>
+          <t>T7</t>
+        </is>
+      </c>
+      <c r="C149" s="9" t="inlineStr">
+        <is>
+          <t>Object-Oriented Programming</t>
+        </is>
+      </c>
+      <c r="D149" s="9" t="inlineStr">
+        <is>
+          <t>topic_7_oop.pdf</t>
+        </is>
+      </c>
+      <c r="E149" s="9" t="inlineStr">
+        <is>
+          <t>Evaluate</t>
+        </is>
+      </c>
+      <c r="F149" s="9" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G149" s="9" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="H149" s="9" t="inlineStr">
+        <is>
+          <t>Best Practice</t>
+        </is>
+      </c>
+      <c r="I149" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J149" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K149" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following Python code that demonstrates method overriding in a single‑inheritance hierarchy:
+```python
+class Base:
+    def greet(self):
+        return "Hello from Base"
+class DerivedA(Base):
+    def greet(self):
+        # Approach 1: explicit base‑class call
+        base_msg = Base.greet(self)
+        return f"{base_msg} and hello from DerivedA"
+class DerivedB(Base):
+    def greet(self):
+        # Approach 2: super() call
+        base_msg = super().greet()
+        return f"{base_msg} and hello from DerivedB"
+```
+Both `DerivedA` and `DerivedB` override `greet` but invoke the base implementation using different techniques. Evaluate which of these two techniques is considered best practice in modern Python for calling a base‑class method, and justify your evaluation by discussing the implications for maintainability, multiple inheritance, and the method resolution order (MRO).</t>
+        </is>
+      </c>
+      <c r="L149" s="9" t="inlineStr">
+        <is>
+          <t>The best‑practice approach is the one used in `DerivedB`, i.e., calling the base method via `super().greet()`. Using `super()` respects Python’s method resolution order, so the call will correctly resolve to the next method in the MRO even when the class participates in multiple inheritance. It also decouples the subclass from the concrete name of its immediate parent, making the code easier to maintain if the inheritance hierarchy changes (e.g., renaming the base class or inserting an intermediate mixin). By contrast, the explicit `Base.greet(self)` call in `DerivedA` bypasses the MRO, works only for single inheritance, and can lead to unexpected behavior or duplicated calls when the class is later used in a multiple‑inheritance scenario. Therefore, `super()` is the recommended, more robust practice.</t>
+        </is>
+      </c>
+      <c r="M149" s="9" t="inlineStr">
+        <is>
+          <t>topic_7_oop.pdf_40, topic_7_oop.pdf_41</t>
+        </is>
+      </c>
+      <c r="N149" s="9" t="inlineStr">
+        <is>
+          <t>Calling base class methods with super()</t>
+        </is>
+      </c>
+      <c r="O149" s="9" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="P107" s="4" t="n"/>
-    </row>
-    <row r="108" customFormat="1" s="8">
-      <c r="A108" s="7" t="inlineStr">
-        <is>
-          <t>T7_020</t>
-        </is>
-      </c>
-      <c r="B108" s="7" t="inlineStr">
+      <c r="P149" s="9" t="n"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="9" t="inlineStr">
+        <is>
+          <t>T7_026</t>
+        </is>
+      </c>
+      <c r="B150" s="9" t="inlineStr">
         <is>
           <t>T7</t>
         </is>
       </c>
-      <c r="C108" s="7" t="inlineStr">
+      <c r="C150" s="9" t="inlineStr">
         <is>
           <t>Object-Oriented Programming</t>
         </is>
       </c>
-      <c r="D108" s="7" t="inlineStr">
+      <c r="D150" s="9" t="inlineStr">
         <is>
           <t>topic_7_oop.pdf</t>
         </is>
       </c>
-      <c r="E108" s="7" t="inlineStr">
+      <c r="E150" s="9" t="inlineStr">
         <is>
           <t>Evaluate</t>
         </is>
       </c>
-      <c r="F108" s="7" t="inlineStr">
+      <c r="F150" s="9" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
       </c>
-      <c r="G108" s="7" t="inlineStr">
-        <is>
-          <t>R4</t>
-        </is>
-      </c>
-      <c r="H108" s="7" t="inlineStr">
+      <c r="G150" s="9" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="H150" s="9" t="inlineStr">
         <is>
           <t>Best Practice</t>
         </is>
       </c>
-      <c r="I108" s="7" t="inlineStr">
+      <c r="I150" s="9" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
       </c>
-      <c r="J108" s="7" t="inlineStr">
+      <c r="J150" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K150" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following Python code that uses a class with an __init__ method but adds an instance attribute outside of it and later deletes it:
+```python
+class MyClass:
+    def __init__(self):
+        self.data = []  # only attribute defined in __init__
+x = MyClass()
+# dynamic attribute creation
+x.counter = 1
+while x.counter &lt; 10:
+    x.counter *= 2
+print(x.counter)
+# attribute removal
+del x.counter
+```
+Evaluate the design choices shown above. Is creating and deleting the `counter` attribute outside `__init__` a good practice? Propose a revised implementation that follows best‑practice guidelines for instance attribute management, and explain why your version is preferable.</t>
+        </is>
+      </c>
+      <c r="L150" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Creating and deleting instance attributes outside of __init__ is generally discouraged. Attributes that are part of an object's state should be declared in __init__ so that every instance starts with a predictable set of members; this improves readability, enables static analysis tools to detect misspellings, and prevents AttributeError at runtime. Dynamically adding `counter` makes the object's interface unclear and forces callers to know that the attribute will exist only temporarily, which violates encapsulation.
+A better design is to define `counter` in __init__ (perhaps with a default value) and encapsulate the loop logic in a method, e.g.:
+```python
+class MyClass:
+    def __init__(self):
+        self.data = []
+        self.counter = 1  # declared up‑front
+    def double_until_limit(self, limit=10):
+        while self.counter &lt; limit:
+            self.counter *= 2
+        return self.counter
+x = MyClass()
+print(x.double_until_limit())
+```
+This version keeps the object's state explicit, avoids the need for `del x.counter`, and makes the behavior reusable and testable. It follows the best‑practice principle that all instance attributes should be initialized in __init__ and manipulated through well‑named methods.
+</t>
+        </is>
+      </c>
+      <c r="M150" s="9" t="inlineStr">
+        <is>
+          <t>topic_7_oop.pdf_23, topic_7_oop.pdf_24, topic_7_oop.pdf_25</t>
+        </is>
+      </c>
+      <c r="N150" s="9" t="inlineStr">
+        <is>
+          <t>Instance attribute initialization best practice</t>
+        </is>
+      </c>
+      <c r="O150" s="9" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="K108" s="4" t="n"/>
-      <c r="L108" s="4" t="n"/>
-      <c r="M108" s="4" t="n"/>
-      <c r="N108" s="4" t="n"/>
-      <c r="O108" s="7" t="inlineStr">
+      <c r="P150" s="9" t="n"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="9" t="inlineStr">
+        <is>
+          <t>T7_027</t>
+        </is>
+      </c>
+      <c r="B151" s="9" t="inlineStr">
+        <is>
+          <t>T7</t>
+        </is>
+      </c>
+      <c r="C151" s="9" t="inlineStr">
+        <is>
+          <t>Object-Oriented Programming</t>
+        </is>
+      </c>
+      <c r="D151" s="9" t="inlineStr">
+        <is>
+          <t>topic_7_oop.pdf</t>
+        </is>
+      </c>
+      <c r="E151" s="9" t="inlineStr">
+        <is>
+          <t>Evaluate</t>
+        </is>
+      </c>
+      <c r="F151" s="9" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G151" s="9" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="H151" s="9" t="inlineStr">
+        <is>
+          <t>Best Practice</t>
+        </is>
+      </c>
+      <c r="I151" s="9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="J151" s="9" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="K151" s="9" t="inlineStr">
+        <is>
+          <t>Consider the following Python code that tries to maintain a shared counter for all instances of a class. The code uses the `global` statement inside a method to modify a module‑level variable.
+```python
+counter = 0
+class Counter:
+    def increment(self):
+        global counter
+        counter += 1
+        return counter
+c1 = Counter()
+c2 = Counter()
+print(c1.increment())  # Expected: 1
+print(c2.increment())  # Expected: 2
+```
+Evaluate this design against the best‑practice guidelines for variable scope discussed in the context. Is using `global` inside the method appropriate for an object‑oriented solution? Propose a revised implementation that follows best practices, and explain why your version is preferable.</t>
+        </is>
+      </c>
+      <c r="L151" s="9" t="inlineStr">
+        <is>
+          <t>Using `global` inside an instance method violates the OOP principle of encapsulation: the method reaches out to a module‑level name instead of managing state that belongs to the class or its instances. The context explains that assignments without a `global` or `nonlocal` statement bind to the innermost (local) scope, and that `global` should only be used when a variable truly belongs in the module namespace. For a shared counter, the idiomatic approach is to store the value as a class attribute, which keeps the state within the class’s own namespace and avoids polluting the module namespace.
+A best‑practice rewrite is:
+```python
+class Counter:
+    _count = 0  # class attribute, shared by all instances
+    def increment(self):
+        Counter._count += 1
+        return Counter._count
+c1 = Counter()
+c2 = Counter()
+print(c1.increment())  # 1
+print(c2.increment())  # 2
+```
+This version uses the class’s namespace (`Counter._count`) to hold the shared state, eliminating the need for `global` and keeping the counter logically tied to the `Counter` class. It follows the guideline that new names are bound in the local scope unless explicitly declared `global` or `nonlocal`, and it respects static name resolution by defining the variable where it conceptually belongs—the class namespace.</t>
+        </is>
+      </c>
+      <c r="M151" s="9" t="inlineStr">
+        <is>
+          <t>topic_7_oop.pdf_14, topic_7_oop.pdf_15, topic_7_oop.pdf_16</t>
+        </is>
+      </c>
+      <c r="N151" s="9" t="inlineStr">
+        <is>
+          <t>Scope Management in OOP</t>
+        </is>
+      </c>
+      <c r="O151" s="9" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="P108" s="4" t="n"/>
-    </row>
-    <row r="109" customFormat="1" s="8">
-      <c r="A109" s="7" t="inlineStr">
-        <is>
-          <t>T7_021</t>
-        </is>
-      </c>
-      <c r="B109" s="7" t="inlineStr">
-        <is>
-          <t>T7</t>
-        </is>
-      </c>
-      <c r="C109" s="7" t="inlineStr">
-        <is>
-          <t>Object-Oriented Programming</t>
-        </is>
-      </c>
-      <c r="D109" s="7" t="inlineStr">
-        <is>
-          <t>topic_7_oop.pdf</t>
-        </is>
-      </c>
-      <c r="E109" s="7" t="inlineStr">
-        <is>
-          <t>Evaluate</t>
-        </is>
-      </c>
-      <c r="F109" s="7" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="G109" s="7" t="inlineStr">
-        <is>
-          <t>R4</t>
-        </is>
-      </c>
-      <c r="H109" s="7" t="inlineStr">
-        <is>
-          <t>Scenario</t>
-        </is>
-      </c>
-      <c r="I109" s="7" t="inlineStr">
-        <is>
-          <t>Mixed</t>
-        </is>
-      </c>
-      <c r="J109" s="7" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="K109" s="4" t="n"/>
-      <c r="L109" s="4" t="n"/>
-      <c r="M109" s="4" t="n"/>
-      <c r="N109" s="4" t="n"/>
-      <c r="O109" s="7" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="P109" s="4" t="n"/>
+      <c r="P151" s="9" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="7">

</xml_diff>